<commit_message>
Add IQOS symbol to hero section from Figma design
Replace placeholder SVG with the real IQOS brand symbol
extracted from the Figma file.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Electric-Dreams-WPP-Creative-Studio.xlsx
+++ b/Electric-Dreams-WPP-Creative-Studio.xlsx
@@ -1,13 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10419"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_0DA30709D718E9450695496250323B1ECBA05575" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="WPP Creative Studio Guide" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Archipelago Sunset Cruise" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Gröna Lund Live Concert" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Floating Sauna Experience" state="visible" r:id="rId7"/>
+    <sheet name="WPP Creative Studio Guide" sheetId="1" r:id="rId1"/>
+    <sheet name="Archipelago Sunset Cruise" sheetId="2" r:id="rId2"/>
+    <sheet name="Gröna Lund Live Concert" sheetId="3" r:id="rId3"/>
+    <sheet name="Floating Sauna Experience" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -169,7 +173,7 @@
     <t>Golden Wake</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A wooden cruise boat glides through the Stockholm archipelago at golden hour. The camera follows from behind, centered on the creamy V-shaped wake that splits the water into two shimmering curtains — one side catching the sinking amber sun, the other side reflecting deep violet sky. Small rocky islands dotted with pine trees drift past in the background. The wake's foam catches pink and lavender highlights. Tracking behind the vessel at water level, drifting slowly upward over 8 seconds to reveal more of the archipelago horizon. Wide — the boat occupies the lower third, the wake fills the middle, and the purple-gold sky dominates the top. The V-shaped wake acts as leading lines that pull the eye toward the violet horizon. Golden hour with clear sky. Warm amber sunlight from the left, filtered through a purple atmospheric haze that tints the shadows indigo. Gold-to-purple gradient on the water surface; deep purple (#2e008b) in the shadows of the islands; soft lavender (#a082e6) in the sky near the horizon; pink (#eb5adc) catching on the foam crests. The boat moves steadily forward; the wake expands rhythmically; gentle ripples propagate outward; distant islands slide past in parallax.</t>
   </si>
   <si>
@@ -191,7 +195,7 @@
     <t>Vaxholm Fortress Pass</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The camera moves laterally along the waterline approaching Vaxholm — the historic gateway to the Stockholm archipelago. The iconic Vaxholm Fortress (Vaxholms kastell) rises on its island in the mid-ground, its stone walls and tower silhouetted against a sky of violet, lavender, and ember-orange. The water between the fortress island and the surrounding granite islets catches fragments of the sky's color — electric violet in the troughs, gold on the wave crests. A thin atmospheric haze softens the town of Vaxholm on the far shore into purple silhouettes layered in depth. Sailing boats are moored near the fortress. Slow lateral dolly at water level, left to right, revealing the fortress and the Vaxholm waterfront in a cinematic parallax. Wide — foreground water detail yields to the sharp fortress mid-ground and a hazy Vaxholm shoreline behind. Vaxholm Fortress as the iconic sentinel of the archipelago — its distinctive stone profile instantly recognizable against the Electric Purple sky. Golden hour with low atmospheric haze. The sun is just off-frame left, casting long warm sidelight that rakes across the fortress walls. Deep purple (#2e008b) on the fortress stone shadows; electric violet (#9b0aa5) on the mid-ground water; soft lavender (#a082e6) in the haze over Vaxholm town; gold and pink (#eb5adc) on the sunlit fortress walls. Gentle lateral drift revealing the fortress from different angles; water laps softly against the fortress island rocks; moored sailboats bob gently; a distant bird glides across the violet sky.</t>
   </si>
   <si>
@@ -210,7 +214,7 @@
     <t>Deck Reflections</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Low-angle shot from deck level of a polished teak boat deck. The wood is wet from sea spray, creating a mirror-like surface that reflects the purple-gold sunset sky above. A coiled nautical rope sits in the left third of frame. The horizon is visible as a thin line of light in the background, out of focus. Warm amber light spills across the deck from the right while purple shadows pool between the planks. Static, positioned just inches above the deck surface, with a very slight forward drift over 8 seconds. Detail — shallow depth of field keeps the nearest planks sharp while the rope and horizon melt into creamy bokeh. The wet deck surface acting as a mirror for the sky's purple-to-gold gradient. Golden hour, dead calm. No wind. The reflection on the deck is almost perfect — a second sky beneath the viewer's feet. Warm amber and soft lavender (#a082e6) reflected on the wet wood; deep purple (#2e008b) in the plank gaps and shadows; pink (#eb5adc) highlights on the rope fibers catching the sun. A single water droplet slides slowly across the polished surface; the reflected clouds drift imperceptibly; the boat sways with the gentlest rocking.</t>
   </si>
   <si>
@@ -232,7 +236,7 @@
     <t>Horizon Melt</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The camera starts just above the water surface — close enough to see individual ripples — then slowly cranes upward to reveal an endless horizon where the dark sea merges with a gradient sky that transitions from deep indigo at the top through electric violet to a thin band of residual amber at the horizon line. A low mist hugs the water surface, diffusing into lavender wisps. The sea is nearly still, with long, slow swells. Slow crane rise — starts at 30cm above water, ends at roughly 3m, maintaining the horizon at the center of frame throughout. Ultra-wide — the horizon line is the subject, stretching edge to edge. The precise line where ocean and sky meet, blurred by mist into an ambiguous, dreamlike boundary. Blue hour, 20 minutes after sunset. The light is cold and ethereal, filtered through a thin mist layer that glows faintly violet. Deep purple (#2e008b) dominating the water and upper sky; electric violet (#9b0aa5) at the horizon glow; soft lavender (#a082e6) in the mist; a whisper of electric blue (#3750dc) in the water highlights. The crane rise is the primary motion; the mist drifts slowly right to left; long ocean swells undulate in slow motion.</t>
   </si>
   <si>
@@ -254,7 +258,7 @@
     <t>Ripple Close-Up</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Extreme close-up of the ocean surface. Each ripple acts as a tiny curved mirror reflecting a different slice of the sunset sky — some crests catch gold, others catch electric violet, others catch pink. The water between the ripples is dark indigo-purple, creating a mosaic of moving color. Occasional micro-bubbles catch the light as tiny pinpoints. Macro lens hovering just above the water surface with a gentle lateral drift, as if floating on the current. Extreme detail — individual ripple crests are razor-sharp; the troughs soften into bokeh. The water surface acting as a fragmented, living canvas of the Electric Purple palette. Golden hour — warm directional light from a low angle creates specular highlights on every ripple crest. Electric violet (#9b0aa5) and gold alternating on ripple crests; deep purple (#2e008b) in the troughs; pink (#eb5adc) specular highlights; light blue (#7da0eb) reflections from the zenith sky. Ripples propagate diagonally across frame in slow motion; light dances across the surface in a hypnotic, rhythmic pattern.</t>
   </si>
   <si>
@@ -276,7 +280,7 @@
     <t>Fjäderholmarna Overhead</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Bird's-eye view looking straight down at a small white cruise boat approaching Fjäderholmarna — the closest archipelago islands to central Stockholm, just 25 minutes from the city. The four small islands of Fjäderholmarna are visible below: Stora Fjäderholmen with its characteristic red wooden buildings and restaurant terraces, the smaller Ängsholmen green with gardens. The water is a deep electric violet, catching lavender and pink highlights where the twilight sky reflects. The boat's wake draws a perfect white line through the purple water, connecting the distant Stockholm skyline (faintly visible at the frame edge) to the island cluster. Top-down drone, slowly rotating clockwise (about 15 degrees over 8 seconds) to add a subtle vertiginous drift. Overhead — the boat is small in frame, emphasizing the island cluster and its relationship to the distant city. Fjäderholmarna as the first taste of the archipelago — the city still visible behind, the wilderness ahead. Twilight — the sky provides even, diffused purple light with no hard shadows. Clear air, no haze. Deep purple (#2e008b) water; electric violet (#9b0aa5) in the open water reflections; the red wooden buildings on Stora Fjäderholmen are warm accents; the boat's white hull is the single bright moving element; wake foam tinted lavender (#a082e6). The boat crawls forward leaving its white wake; the drone rotates slowly; tiny ripples spread outward from the boat's passage; lights begin to glow on the island terraces.</t>
   </si>
   <si>
@@ -298,7 +302,7 @@
     <t>Bow Spray</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Shot from the bow of the boat, looking forward and slightly down. The prow cuts through the water, sending up curtains of fine spray on both sides. The spray is backlit by the setting sun, turning each droplet into a tiny prism of gold, violet, and pink. Through the spray, the purple horizon and distant islands are visible but softened. The polished brass fitting on the bow catches a warm purple-gold reflection. Low-angle, mounted near the waterline on the bow, with a subtle forward lean as the boat rises and dips on gentle swells. Medium — the spray curtain is the sharp subject; the horizon beyond is soft and dreamy. Backlit spray droplets acting as prisms for the Electric Purple palette. Sunset with strong backlight. The sun is low and directly ahead, creating a corona effect filtered through the spray. Gold and pink (#eb5adc) in the backlit spray; electric violet (#9b0aa5) in the water; deep purple (#2e008b) in the shadowed hull; soft lavender (#a082e6) in the sky beyond. Continuous spray arcing upward and falling back; the boat rocks gently on swells; droplets hang in slow motion mid-air.</t>
   </si>
   <si>
@@ -320,7 +324,7 @@
     <t>Lantern Glow</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A string of warm Edison-bulb lanterns stretches across the boat's deck, their amber glow creating pools of warm light on the wooden surface. Beyond the deck railing, the blue-hour sky is a deep electric violet gradient. The lanterns' light reflects on polished brass fittings and glass surfaces on deck. A wine glass sits on a small table, catching both the amber lantern light and the violet sky. Slow orbit around the lantern string, moving roughly 30 degrees over 8 seconds, keeping the lights and sky in constant relationship. Medium — the nearest lantern bulb is in focus with creamy bokeh on the more distant bulbs and the purple sky. The warm amber of the lanterns against the cold violet of the twilight sky — a temperature contrast that unifies in the Electric Purple palette. Blue hour — the sky is luminous violet-blue; the deck is lit only by the practical lanterns. Warm amber/gold from lanterns; deep purple (#2e008b) sky; electric violet (#9b0aa5) at the horizon; soft lavender (#a082e6) bokeh on distant lights; the wine glass catches pink (#eb5adc) reflections. Slow orbital drift; lanterns sway gently with the boat's rocking; the wine glass surface trembles with micro-ripples.</t>
   </si>
   <si>
@@ -339,7 +343,7 @@
     <t>Sail Silhouette</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A classic wooden sailboat in perfect silhouette against a sky that bleeds from deep amber at the horizon through electric violet to deep purple overhead. The sails are full but the boat moves slowly — the scene is about stillness, not speed. The water below is a dark mirror, reflecting the sky's gradient in muted, deeper tones. A few small islands sit on the horizon as dark shapes. Static wide shot. The boat is positioned at the rule-of-thirds intersection, left third of frame. No camera movement — the stillness is the point. Wide — everything from the water's edge to the clouds is in focus, creating a painterly depth. The stark black silhouette of the sailboat's mast, rigging, and hull against the intensely colored sky. Peak sunset — the sky is at maximum saturation. No clouds, just pure gradient. The sky is the canvas — amber at bottom, electric violet (#9b0aa5) in the middle, deep purple (#2e008b) at the top. The water mirrors this but two stops darker. The silhouette is pure black (#34303d). Minimal — the boat drifts almost imperceptibly; the water surface shimmers with slow, oily undulations; the reflected colors shift subtly.</t>
   </si>
   <si>
@@ -358,7 +362,7 @@
     <t>Northern Shimmer</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Late Nordic summer night — the sky never fully darkens. The camera starts on the dark silhouettes of archipelago islands reflected in still water, then tilts slowly upward to reveal a sky where the deep purple of night is interrupted by faint, shimmering curtains of green-tinted aurora, interweaving with the dominant violet and lavender tones. Stars are faintly visible. The water below mirrors both the aurora and the purple sky. Slow tilt up — starts on water reflection, ends on the aurora-tinged sky. Steady, meditative pace. Wide — sharp from the island silhouettes to the stars. The rare interplay of faint aurora greens woven into the Electric Purple palette — a uniquely Nordic phenomenon. Clear Nordic summer night. The air is perfectly still. The temperature of the light is cold but alive with subtle color shifts. Deep purple (#2e008b) as the base sky; electric violet (#9b0aa5) and soft lavender (#a082e6) in the aurora curtains (with faint green accents); electric blue (#3750dc) in the star reflections on water. The tilt is the primary motion; the aurora shimmers in slow, undulating curtains; stars twinkle subtly; water reflects everything in gentle distortion.</t>
   </si>
   <si>
@@ -377,7 +381,7 @@
     <t>Wave Texture</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The camera travels alongside the boat at water level, focused on the ocean surface texture as it reacts to the hull's passage. The water has a deep electric violet base color with golden-hour light painting every wave crest in amber. The interaction between the hull's pressure wave and the open sea creates complex, mesmerizing patterns — standing waves, interference patterns, and tiny vortices. Tracking alongside the hull at water level, matching the boat's speed, focused on the 2-meter zone where hull meets water. Detail — the nearest wave textures are sharp; background water softens into an impressionist blur of violet and gold. The complex fluid dynamics of water against hull, painted in purple and gold. Golden hour — low-angle sunlight rakes across the wave texture, exaggerating every crest and trough with dramatic light and shadow. Electric violet (#9b0aa5) in the wave troughs and shadows; gold crests; deep purple (#2e008b) in the deeper water; occasional pink (#eb5adc) highlight where spray catches direct sun. Continuous forward tracking; complex fluid motion in the wave patterns; occasional spray droplets arcing through frame.</t>
   </si>
   <si>
@@ -393,7 +397,7 @@
     <t>Landsort Lighthouse</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Dusk settling over the southernmost point of the Stockholm archipelago. The historic Landsort lighthouse — Sweden's oldest still-operating lighthouse, built in 1689 — stands on its rocky island of Öja, its distinctive white tower emitting a rotating beam that cuts through a low-hanging violet mist. Each sweep of the beam illuminates the mist in a cone of soft lavender light before fading. The rugged, windswept rocks of Landsort's southern tip frame the shot in the foreground. The open Baltic Sea stretches beyond, its surface glassy and reflecting the lighthouse beam as a shimmering purple stripe. The cluster of red wooden pilot houses at the base of the lighthouse adds warm accent. Slow dolly forward across the open water, approaching Landsort island over 8 seconds. Wide — foreground wave crests are soft; the lighthouse tower and its beam are the mid-ground subject; the open Baltic horizon is ultra-soft in fog. The Landsort lighthouse as the archipelago's outermost sentinel — where Sweden meets the open sea, its historic beam sweeping through purple twilight. Twilight with dense low fog rolling in from the Baltic. Visibility is limited, creating a mysterious, edge-of-the-world feeling. Soft lavender (#a082e6) in the illuminated mist cone; deep purple (#2e008b) in the surrounding darkness; electric violet (#9b0aa5) on the water reflection of the beam; the white lighthouse tower catches purple ambient light; warm red from the pilot houses. Slow forward dolly; the lighthouse beam sweeps once fully across frame during the 8 seconds; mist drifts and swirls in the beam's wake; Baltic waves roll against the rocky shore.</t>
   </si>
   <si>
@@ -412,7 +416,7 @@
     <t>Sunset Burst</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The exact moment the sun touches the horizon line. The sky detonates into bands of color — amber closest to the sun, then hot pink, electric violet, soft lavender, and finally deep purple overhead. Thin clouds catch these colors and streak them horizontally across the frame. The sea below is a dark mirror reflecting the explosion in slightly muted tones. A few island silhouettes punctuate the horizon. Static — locked off on a tripod. The stillness contrasts with the sky's intensity. Very subtle exposure shift as the sun moves. Wide — everything sharp, horizon to zenith. The sun itself at the exact moment of horizon contact, with the sky as a full-spectrum showcase of the Electric Purple palette. Peak sunset — maximum color saturation. Clear sky with scattered high cirrus clouds acting as color canvases. Full palette in natural gradient — amber/gold at the center, pink (#eb5adc), electric violet (#9b0aa5), soft lavender (#a082e6), deep purple (#2e008b) radiating outward. Near-static — the sun sinks imperceptibly; clouds drift at altitude; the sea surface catches and releases colors in slow, breathing undulations.</t>
   </si>
   <si>
@@ -431,7 +435,7 @@
     <t>Rope &amp; Rail</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Close-up of a coil of thick nautical rope resting on a brass rail at the side of the boat. The rope's hemp fibers catch warm golden-hour light, revealing texture and subtle purple shadow between the coils. Behind the railing, the archipelago water is a field of purple and gold bokeh circles. The brass rail has a warm amber patina with violet reflections from the sky. Slow pan from the rope coil to the right, gradually shifting focus from the rope to the water beyond the railing. Detail — shallow depth of field. The rope starts sharp, then focus racks to the water bokeh, then back. The tactile materiality of the rope — hemp, brass, wood — juxtaposed with the ethereal purple bokeh of the sea. Golden hour, calm. Warm sidelight from the left paints the rope in amber while the shadows between coils are deep violet. Warm amber on rope fibers; deep purple (#2e008b) shadows; soft lavender (#a082e6) and pink (#eb5adc) bokeh circles on the water; brass rail reflects electric violet (#9b0aa5) from the sky. Slow pan; the rope sways almost imperceptibly with the boat's gentle rocking; bokeh circles on the water shift and dance.</t>
   </si>
   <si>
@@ -447,7 +451,7 @@
     <t>Sandhamn Passage</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The boat enters the iconic narrow passage approaching Sandhamn — the legendary sailing destination in the outer Stockholm archipelago. The camera is positioned at the bow, looking forward through the gap between Sandön and the neighboring island. The distinctive yellow and red wooden houses of Sandhamn village are visible at the far end of the strait, their facades catching the golden-hour light. The islands rise on either side with weathered granite cliffs and wind-shaped pines silhouetted against the purple-gold sky. The water in the strait is calm and deeply colored — almost black-purple in the cliff shadows, brightening to violet where the sky light reaches it. Classic wooden sailing yachts are moored along the Sandhamn waterfront. Slow dolly forward, as if riding the bow of the boat through the narrows into Sandhamn. The village slowly reveals itself as the boat progresses. Wide — sharp cliff faces on either side framing the village ahead. Sandhamn as the archipelago's most celebrated destination — its colorful wooden village emerging from between the dark rock walls like a hidden jewel. Golden hour with atmospheric haze diffusing the light around the village. The warm light on the old wooden facades contrasts with the purple shadows of the narrows. Deep purple (#2e008b) and near-black on the cliff faces; electric violet (#9b0aa5) on the water surface; warm gold and amber on the Sandhamn village facades; soft lavender (#a082e6) haze around the village; the classic sailing boats' white hulls catch pink (#eb5adc) light. Forward dolly through the narrows; water ripples reflect off the cliff walls; moored boats rock gently; the village grows larger and more detailed as the boat approaches.</t>
   </si>
   <si>
@@ -463,7 +467,7 @@
     <t>Glass Surface</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The camera skims just millimeters above a perfectly still water surface that mirrors the blue-hour sky so faithfully that it is nearly impossible to tell where water ends and sky begins. The reflected sky is a deep gradient from electric violet at the horizon to deep purple overhead. A single island silhouette appears both above and below the waterline in perfect symmetry. The only disruption is one tiny ripple that slowly expands from where a raindrop fell. Low-angle skim — the lens is nearly touching the water surface, drifting forward with infinite slowness. Detail — the single expanding ripple is sharp; the reflected sky and island are slightly soft. The perfect mirror symmetry between water and sky, disrupted by one poetic ripple. Blue hour, dead calm. No wind, no waves. The world feels held in suspension. Electric violet (#9b0aa5) at the mirror horizon; deep purple (#2e008b) in both the real and reflected sky; soft lavender (#a082e6) in the ripple's interference pattern; electric blue (#3750dc) at the zenith and its reflection. Near-static — the single ripple expands in concentric rings; the camera drifts almost imperceptibly forward; the island reflection shimmers.</t>
   </si>
   <si>
@@ -482,7 +486,7 @@
     <t>Cloud Cathedral</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Starting on the dark purple water surface, the camera tilts upward to reveal a cathedral of cumulonimbus clouds rising into the upper atmosphere. The clouds are lit from below by the setting sun — their bases glow amber and electric violet, while their towering tops darken to deep indigo-purple. Light shafts break through gaps between clouds, striking the water as lavender god-rays. A thin strip of orange horizon is visible between the water and the cloud base. Slow tilt up — water to sky, taking the full 8 seconds to reveal the clouds' full height. Wide — deep focus from the water surface through to the cloud tops. The monumental scale of the cloud formations lit in the Electric Purple palette, creating a natural cathedral. Sunset with dramatic cloud cover. Volumetric light beams. The air feels heavy with potential. Deep purple (#2e008b) in the cloud tops and water; electric violet (#9b0aa5) on the cloud bases; soft lavender (#a082e6) in the god-rays; pink (#eb5adc) on the cloud edges catching direct sunset light. Slow tilt upward; clouds billow and evolve in slow motion; god-rays shift and breathe; the water surface catches falling light patches.</t>
   </si>
   <si>
@@ -501,7 +505,7 @@
     <t>Wake Symmetry</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Drone view following directly above and behind a cruise boat. The vessel creates a perfect symmetrical V-wake that stretches to the bottom of frame and beyond. The wake's white foam lines create a strong geometric pattern against the deep violet water. Golden-hour light catches the wake's outer edges in amber while the inner water between the V is sheltered and darker purple. Tiny islands are scattered across the seascape ahead. Following drone at about 50m altitude, locked onto the boat, maintaining the V-wake centered in frame. Overhead — the geometric wake pattern is the composition. The mathematical perfection of the V-wake as a graphic element drawn in white on a purple canvas. Golden hour — directional light from the left creates a warm/cool split on the wake: left side amber-lit, right side in purple shadow. Deep purple (#2e008b) water; white wake foam with lavender (#a082e6) tint in the shadow side; electric violet (#9b0aa5) in the wider water; golden amber on the sun-facing wake edge; islands as dark spots. Steady forward following; the wake continuously unfurls; small boats or markers pass below in parallax; water texture ripples.</t>
   </si>
   <si>
@@ -517,7 +521,7 @@
     <t>Möja Midnight Sun</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The Nordic midnight sun hangs just above the horizon, refusing to set, viewed from the eastern shore of Möja — one of the largest and most beloved islands in the outer Stockholm archipelago. The distinctive Möja landscape is visible: the rocky eastern shoreline with its smooth, glacier-polished granite slabs, a few weathered red fishing huts (sjöbodar) along the shore, and the sparse pine forest silhouetted behind them. The sky is a perpetual twilight gradient — amber at the horizon, cycling through electric violet to deep purple overhead. The entire 360-degree sky glows. The open Baltic water beyond Möja reflects this wrap-around light, creating an otherworldly scene where everything is suffused in purple-gold. Fishing nets and lobster pots on the shore add texture. Static ultra-wide. The horizon bisects the frame perfectly. No movement — the scene's strangeness speaks for itself. Ultra-wide — the entire panoramic scene from Möja's shore to the distant horizon is in focus. The midnight sun viewed from Möja's raw outer-archipelago landscape — where the comfort of the village meets the wildness of the open Baltic. Nordic midnight sun — a quality of light that exists nowhere else. Neither day nor night. Temperature neutral, tending purple. Equal balance of amber and purple — electric violet (#9b0aa5) in the mid-sky, deep purple (#2e008b) at zenith, soft lavender (#a082e6) in the water reflections, gold at both horizons; warm red on the fishing huts. Extremely minimal — the sun barely moves along the horizon; water shimmers against the smooth granite; a flag on a fishing hut barely stirs.</t>
   </si>
   <si>
@@ -533,7 +537,7 @@
     <t>Anchor Drop</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The anchor chain runs taut from the boat's bow downward into deep purple water. The camera follows it, tilting slowly downward. Where the chain enters the water, a column of silver-white bubbles rises, backlit by the last purple-amber light from the sky. The chain disappears into the depths, which darken from electric violet to pure indigo-black. The underwater portion shows the chain slightly refracted and wavering. Slow downward tilt following the chain from deck level into the water. The transition from above-water to below-water happens at roughly the 4-second mark. Medium — the chain is the sharp subject; the water surface and the depths beyond are soft. The chain as a connector between the world above (amber-lit) and the world below (deep purple) — a vertical journey through the palette. Dusk — the last light catches the chain and bubbles while the water below is already immersed in deep purple darkness. Amber on the dry chain above water; deep purple (#2e008b) in the depths; electric violet (#9b0aa5) at the waterline; soft lavender (#a082e6) in the bubbles; light blue (#7da0eb) refracted through the water surface. The chain runs slowly downward; bubbles rise and wobble; the water surface undulates from above, then closes over the camera's perspective.</t>
   </si>
   <si>
@@ -552,7 +556,7 @@
     <t>Grinda Birch Shore</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The camera moves past a cluster of white birch trees on Grinda island — one of the most popular nature islands in the inner archipelago, known for its lush deciduous forests. The pale birch trunks and trembling green-gold leaves act as natural frames for the scene beyond: a purple sea stretching toward the distant silhouettes of Viggsö and Svartsö islands, with a cruise boat passing in the mid-ground. Grinda's iconic meadow landscape is hinted at through the trees — wild flowers at the base of the birches. The birch bark catches warm golden light while the spaces between the trunks reveal the deep violet water. Lichen-covered granite rocks typical of Grinda's shoreline anchor the foreground. Slow dolly laterally, passing behind and between birch trunks in a smooth parallax. The boat appears and disappears between the trunks. Layered — foreground birch trunks are sharp, mid-ground water is in focus, distant island silhouettes are slightly soft. Grinda's lush birch forest as a natural cinema screen — the white trunks framing slices of the purple seascape in a composition unique to this island's character. Golden hour — warm sidelight on the birch bark, purple shadow between the trees. The combination is iconic Swedish summer. White-silver birch bark catching gold and pink (#eb5adc) light; deep purple (#2e008b) sea visible between trunks; soft lavender (#a082e6) sky; electric violet (#9b0aa5) in the tree shadows; meadow wildflowers adding tiny purple and yellow accents at the base. Lateral dolly creating parallax between tree layers; birch leaves tremble in a light breeze; the distant boat glides smoothly; a butterfly crosses the foreground meadow flowers.</t>
   </si>
   <si>
@@ -571,7 +575,7 @@
     <t>Foam Trail</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Extreme close tracking shot of the boat's wake foam. The churning white-lavender foam contrasts sharply with the deep violet water surrounding it. Sunset backlight penetrates the thinner foam sections, turning them translucent pink and gold. Air bubbles trapped in the foam catch individual specular highlights. As the foam dissipates at the edges, it transitions from white to lavender to deep purple water in a beautiful gradient. Tracking close alongside the wake, matching the boat's speed, focused on the foam texture roughly 1 meter from the hull. Detail — the foam texture is razor-sharp; the water beyond falls to soft purple bokeh. The ephemeral beauty of sea foam — its white chaos against the controlled deep purple of the water. Sunset backlight — every bubble and foam strand is edge-lit in gold and violet. White foam with lavender (#a082e6) tint in shadows; deep purple (#2e008b) water; pink (#eb5adc) and gold in backlit translucent foam; electric violet (#9b0aa5) where foam dissolves into water. Continuous tracking; the foam churns and evolves organically; bubbles pop and reform; the edge between foam and water is constantly negotiated.</t>
   </si>
   <si>
@@ -587,7 +591,7 @@
     <t>Dalarö Panorama</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A sweeping 180-degree panoramic view from the historic harbor of Dalarö — the southern gateway to the Stockholm archipelago since the 17th century. The camera slowly pans from west (where the last amber glow clings to the horizon above the Dalarö skans fortress ruins) through south (the open water toward Ornö and Utö, pure electric violet sky) to east (where the sky deepens to indigo above the small islands of the Dalarö archipelago). The distinctive Dalarö waterfront is visible in the pan — traditional red and yellow wooden houses along the harbor, historic steamboat pier, and classic archipelago boats moored in a row. Dozens of islands are scattered across the southern view at varying distances, each a different shade of purple silhouette. Slow 180-degree pan, smooth and steady, completing the sweep in 8 seconds. Eye-level from the Dalarö harbor pier. Ultra-wide — maximizing the panoramic depth from the harbor foreground to the distant island layers. Dalarö as the meeting point between historic maritime culture and wild archipelago nature — its charming harbor opening onto the vast purple seascape. Blue hour — the light is even, cool, and deeply violet. No hard shadows. The air is crystalline. Full purple gradient — from residual amber/gold in the west, through electric violet (#9b0aa5), to deep purple (#2e008b) in the east. Warm red and yellow Dalarö facades add color contrast; islands layer in progressively lighter purple — dark indigo nearest, soft lavender (#a082e6) farthest. Continuous smooth pan; harbor boat lights blink; water shimmers differently at each compass point; the Swedish flag on the steamboat pier sways gently.</t>
   </si>
   <si>
@@ -603,7 +607,7 @@
     <t>Mast &amp; Stars</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Starting on the warm-lit wooden deck, the camera tilts slowly upward along the boat's mast. The mast is a dark vertical line that bisects the frame, its rigging lines radiating outward like a spider's web. As the camera rises, it passes through the deck-light zone (warm amber) into the middle zone (electric violet sky) and finally into the upper sky (deep purple with the first visible stars). The mast's peak has a small amber navigation light that acts as a warm counterpoint to the cold stars. Slow tilt upward, following the mast from deck to sky tip over 8 seconds. The mast stays centered throughout. Vertical composition — the bottom is detail (deck texture), the middle is medium (rigging), the top is wide (open sky with stars). The mast as a vertical axis connecting earth (deck) to cosmos (stars), transitioning through the full Electric Purple palette. Night onset — the deck retains warm practical light while the sky has fully shifted to purple. Stars are just appearing. Warm amber at the deck base; electric violet (#9b0aa5) in the mid-sky; deep purple (#2e008b) at the zenith; soft lavender (#a082e6) in the star glow; the navigation light is a warm amber jewel. Slow upward tilt; the rigging lines sway gently; stars flicker; the navigation light glows steadily; the mast itself sways with the boat's rock.</t>
   </si>
   <si>
@@ -625,7 +629,7 @@
     <t>Last Light over Utö</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The very last sliver of the sun disappears behind the silhouette of Utö — the southernmost inhabited island in the Stockholm archipelago, recognizable by the profile of its historic windmill and the old mining village skyline. For a brief moment, the windmill and the island's ridge are rimmed in blinding gold — a thin line of fire separating the dark landmass from the purple sky. The sky above Utö glows in a diminishing aureole of amber that fades rapidly through pink into electric violet and finally deep purple. The water catches the last reflection — a single golden path that narrows and darkens as the sun vanishes. The small harbor lights of Gruvbryggan (Utö's main pier) twinkle at the base of the silhouette. Slow zoom out — starting tight on the sun-rimmed windmill silhouette, widening to reveal Utö's full profile against the purple sky. Wide — the rim-light edge is sharp; the expanding view stays in focus to communicate the vastness of the moment. Utö's iconic windmill silhouette as the last point where sunlight touches the archipelago — a recognizable landmark marking the end of the day and the southernmost reach of the island chain. Sunset end — the transition point between golden hour and blue hour. The light is fading rapidly and the purple is winning. Intense gold/amber rim on the windmill and island edge; pink (#eb5adc) aureole closest to the sun; electric violet (#9b0aa5) expanding outward; deep purple (#2e008b) overtaking the sky; soft lavender (#a082e6) in the fading water reflection; warm harbor lights as tiny amber points. Slow zoom out; the golden rim thins and extinguishes; the purple expands to fill the frame; the water reflection narrows to a point; harbor lights grow more visible as the natural light fades.</t>
   </si>
   <si>
@@ -650,7 +654,7 @@
     <t>Stage Pulse</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A massive outdoor concert stage at Gröna Lund, seen from the back of the crowd. The stage is a wall of deep purple and electric violet light, pulsing rhythmically with a bass-heavy beat. Theatrical haze fills the air, catching the light beams and turning them into solid cones of violet. The stage's LED screens display abstract purple wave patterns. Silhouettes of the crowd's raised hands fill the lower third of frame. Slow dolly forward through the crowd — as if pushing toward the stage. The stage grows larger and more intense over 8 seconds. Wide — the stage is the subject, the crowd silhouettes frame it. The stage as a monolithic source of purple light, radiating energy outward through the haze. Night with heavy theatrical haze. The air is thick with light beams made visible by the fog. Every breath catches violet. Electric violet (#9b0aa5) as the dominant stage wash; deep purple (#2e008b) in the sky and shadows; pink (#eb5adc) accent lights; soft lavender (#a082e6) in the haze; the crowd is near-black silhouette. Forward dolly; haze drifts and swirls; light beams pulse with the rhythm; crowd hands sway; stage LEDs animate.</t>
   </si>
   <si>
@@ -669,7 +673,7 @@
     <t>Neon Ferris &amp; Gamla Stan</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The iconic Gröna Lund ferris wheel dominates the frame, its structure outlined in LED lights cycling through the Electric Purple palette — from deep purple at the base through electric violet on the spokes to soft lavender at the top. Each gondola has a pink accent light. As the camera orbits, the Stockholm skyline reveals itself behind the wheel — the unmistakable silhouette of Gamla Stan (the Old Town) with its church spires and the Royal Palace is visible across the dark harbor water, bathed in warm amber light that contrasts with the purple night sky. The Djurgården waterfront below glitters with the park's reflected neon. Slow orbit — the camera circles the ferris wheel about 30 degrees over 8 seconds, shifting the Gamla Stan skyline from hidden to revealed behind the wheel. Wide — the full ferris wheel in frame with Gamla Stan's silhouette and harbor reflections. The ferris wheel as a giant purple mandala with Stockholm's most historic quarter visible through its spokes — modern spectacle framing centuries of history. Night, clear sky. The ferris wheel is the brightest object in frame, with Gamla Stan's warm glow as the atmospheric backdrop. Electric violet (#9b0aa5) on the wheel structure; deep purple (#2e008b) sky; pink (#eb5adc) gondola accents; warm amber on Gamla Stan's facades; soft lavender (#a082e6) light spill; electric blue (#3750dc) harbor water reflections bridging Djurgården to the Old Town. The ferris wheel rotates slowly; gondolas sway; the orbit reveals Gamla Stan progressively; LED lights animate in sequence; harbor reflections of both park and Old Town shimmer.</t>
   </si>
   <si>
@@ -685,7 +689,7 @@
     <t>Bass Drop</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A massive wall of black speaker stacks at the side of the stage. The camera faces them straight-on, close enough to feel the vibration. The speaker cones pulse visibly with each bass hit. The air in front of the speakers distorts like heat haze — visible compression waves. Purple and violet stage light bathes the speaker cabinets from behind, creating a dramatic rim-light on their edges. A thin layer of mist at the base catches the light. Static with subtle physical shake synchronized to the bass hits — the camera itself vibrates with the sound pressure. Medium — the speaker wall fills the frame; individual cone movements are visible. The raw physical power of sound made visible — vibrating cones, air distortion, camera shake. Night, intense. The bass is felt more than heard. The air itself seems to pulse purple. Deep purple (#2e008b) on the speaker cabinets; electric violet (#9b0aa5) rim-light from behind; soft lavender (#a082e6) in the mist at the base; occasional pink (#eb5adc) flash from stage effects. Speaker cones pulse rhythmically; visible air compression waves; camera micro-shakes on each bass hit; mist at the base ripples with the pressure waves.</t>
   </si>
   <si>
@@ -704,7 +708,7 @@
     <t>Laser Cathedral</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Looking upward from the crowd level as dozens of laser beams cut through dense fog above the stage. The lasers create a geometric grid — parallel lines, fans, and cones — in electric violet, pink, and soft lavender. Where the beams intersect, they create brighter nodes of light. The fog is thick enough to make each beam a solid line of light. Through the laser grid, the dark purple night sky is faintly visible. Tilt up — starting from the crowd's raised hands, ascending through the laser grid to the open sky over 8 seconds. Wide — the entire laser architecture is in view, creating a cathedral of light. The geometric precision of laser beams contrasting with the organic movement of fog — order and chaos in purple light. Night with very heavy theatrical fog. The lasers need the fog to exist visibly — they are painting on a canvas of mist. Electric violet (#9b0aa5) primary lasers; pink (#eb5adc) accent lasers; soft lavender (#a082e6) where beams scatter in the fog; deep purple (#2e008b) in the negative space between beams. Lasers sweep slowly in synchronized patterns; fog drifts and curls around the beams; beam intersections pulse; the tilt reveals new layers of the laser architecture.</t>
   </si>
   <si>
@@ -723,7 +727,7 @@
     <t>Confetti Rain</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Thousands of pieces of confetti in shades of purple, violet, lavender, and pink fall through the air in extreme slow motion. Each piece tumbles and rotates, catching spotlight beams from different angles — sometimes opaque and dark, sometimes translucent and glowing. The confetti is in sharp focus in the mid-ground while the background stage lights are soft purple bokeh circles. Occasional gold confetti pieces provide warm accent. Slow-motion capture of the confetti fall, with a very slight downward drift matching the confetti's trajectory. Detail — individual confetti pieces are readable; some are so close they're large abstract shapes passing through the foreground bokeh. The confetti as individual carriers of the Electric Purple palette — each piece a tiny canvas. Night, celebratory peak moment. The confetti cannon has just fired. The air is full of color. Every piece is a different shade — deep purple (#2e008b), electric violet (#9b0aa5), soft lavender (#a082e6), pink (#eb5adc), with gold accents. The background bokeh is electric violet. Ultra-slow-motion tumble of confetti; each piece rotates and catches light at different angles; some pieces collide and redirect; spotlight beams illuminate different zones.</t>
   </si>
   <si>
@@ -742,7 +746,7 @@
     <t>Crowd Silhouettes</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A wide shot of the concert crowd in complete silhouette. The stage behind them is a solid wall of purple-violet light with horizontal bands of intensity — brightest at center, darkening to the edges. The crowd forms a jagged horizon line of dark shapes — raised hands, phones, shoulders, heads — all anonymous and unidentifiable. Occasional wisps of haze drift between the camera and the crowd, catching purple light. Static wide — locked off. The power of the image comes from the graphic simplicity of black silhouettes against purple. Wide — the silhouette edge is crisp where dark meets light. The crowd as a collective abstract shape — a mountain range of human energy, defined only by its outline against the purple light. Night — the only light source is the stage. The relationship between the dark crowd mass and the purple light is the entire image. The stage wash blends electric violet (#9b0aa5) at center with deep purple (#2e008b) at edges; the crowd is pure dark (#34303d) silhouette; stray haze catches soft lavender (#a082e6); phone screens are tiny dots of light blue (#7da0eb). Minimal — hands sway slowly; occasional phone screens light up and dim; haze drifts languidly across the frame; the stage light breathes slightly with the music.</t>
   </si>
   <si>
@@ -761,7 +765,7 @@
     <t>Guitar Strings</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Extreme macro of an electric guitar's strings, seen from the side. The strings vibrate with visible standing-wave patterns — each string a blur of harmonic motion. Purple and violet stage light catches on the chrome frets and wound string surfaces. A lens flare from a distant spotlight bleeds across the frame in soft lavender and pink. The guitar body beyond the strings is dark wood catching purple rim light. Macro drift — slowly panning from the low strings to the high strings over 8 seconds, maintaining extreme close focus. Extreme detail — the strings' vibration blur is the subject; the guitar body beyond is soft bokeh. Sound made visible — the strings' vibration patterns are a physical manifestation of music. Night, intimate — this is a private view of the instrument. The macro perspective makes the guitar a landscape. Chrome and silver strings catching electric violet (#9b0aa5) light; deep purple (#2e008b) in the shadows between strings; soft lavender (#a082e6) and pink (#eb5adc) in the lens flare; warm amber on the wood body. The strings vibrate at different frequencies — visible standing waves; the camera drifts slowly across them; lens flare shifts with the camera position; light reflections dance on the chrome frets.</t>
   </si>
   <si>
@@ -780,7 +784,7 @@
     <t>Spotlight Sweep</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A single powerful spotlight beam sweeps slowly across the venue, cutting a solid cone of lavender-white light through the purple haze. Everything the beam touches is momentarily illuminated — truss structures, rigging cables, the upper reaches of the crowd — before falling back into purple darkness. The beam's edges are soft and feathered by the haze. Where it hits the haze densely, it blooms into a soft, volumetric lavender cloud. Tracking the beam — the camera follows the spotlight's sweep, keeping the brightest point centered in frame as it moves across the venue. Wide — the beam and its interaction with the architecture and haze. The spotlight beam as a physical object — a solid bar of light that reveals and conceals as it sweeps. Night with medium haze. The beam is only visible because of the particulates in the air. The surrounding darkness is deep purple. White-lavender (#a082e6) in the beam core; electric violet (#9b0aa5) at the beam edges where it diffuses; deep purple (#2e008b) in the negative space; momentary pink (#eb5adc) where the beam hits colored surfaces. The beam sweeps in a smooth arc; haze swirls in its wake; the camera tracks with the beam; particles in the air sparkle as they pass through the beam.</t>
   </si>
   <si>
@@ -796,7 +800,7 @@
     <t>Drum Hit</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Ultra-slow-motion capture of a drumstick striking a cymbal. The impact sends a visible shockwave across the cymbal's surface — concentric ripples propagating outward from the strike point. Tiny droplets of condensation fly off the cymbal in a crown pattern. Purple and violet stage light reflects off the cymbal's bronze surface in shifting, liquid patterns. The stick rebounds in a graceful arc, trailing a slight motion blur. Slow-motion, positioned at cymbal level, capturing the impact from a 45-degree angle. Detail — the strike point is razor-sharp; the cymbal edges blur with motion; the background is pure purple bokeh. The violence and beauty of percussion — a single strike as a universe of physics and light. Night, dynamic. Stage lighting from above and behind catches the cymbal as a reflective surface for the purple palette. Bronze cymbal reflecting electric violet (#9b0aa5) and amber; deep purple (#2e008b) background; soft lavender (#a082e6) in the flying droplets; pink (#eb5adc) reflected in the concentric waves. Ultra-slow-motion: the stick's impact, the wave propagation, the droplet crown, the rebound arc — all happening in dreamy time.</t>
   </si>
   <si>
@@ -815,7 +819,7 @@
     <t>Djurgården Skyline</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The camera rises on a crane above Gröna Lund on Djurgården island, revealing the full park skyline and the sweeping Stockholm panorama beyond. Roller coaster tracks, the ferris wheel, swing rides, and tower rides are all outlined in colored lights. As the crane ascends, Stockholm's most iconic landmarks reveal themselves: to the left, the grand boulevard of Strandvägen with its Art Nouveau facades and moored vintage boats; across the water, the distinctive silhouette of Stockholm City Hall (Stadshuset) with its three golden crowns tower; further left, the spires of Gamla Stan; and the Nordiska Museet's Renaissance castle silhouette right next to the park. The harbor water reflects the entire spectacle in shimmering purple. Crane rising — starting at crowd level, ascending to reveal the full Djurgården-to-city panorama over 8 seconds. Slow, majestic ascent. Ultra-wide — the entire park, harbor, and Stockholm skyline in one frame. Gröna Lund's position on Djurgården revealed as central to Stockholm's most beautiful waterfront — the park as the electric heart of the city's cultural island. Night, clear. The sky has that deep electric purple that clean Nordic air produces after dark, with Stockholm's light pollution creating a lavender dome over the city. Electric violet (#9b0aa5) LED lights on rides; deep purple (#2e008b) night sky; pink (#eb5adc) neon accents; Strandvägen and Stadshuset in warm amber; soft lavender (#a082e6) light pollution dome; electric blue (#3750dc) harbor reflections connecting park to city. The crane rises steadily; ride lights animate; the ferris wheel rotates; the expanding view reveals more of Stockholm's waterfront; harbor reflections dance.</t>
   </si>
   <si>
@@ -831,7 +835,7 @@
     <t>Strobe Freeze</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The stage strobes fire in rapid succession, and the camera captures the moments between flashes — frozen tableaux of the scene lit only by the persistent purple wash. Each strobe flash reveals a slightly different composition: haze has moved, light beams have shifted, confetti has fallen further. Between flashes, the scene is a deep purple low-light painting where only the brightest elements (LED panels, reflective surfaces) are visible. Strobe-cut style — simulating the visual effect of being in a strobe environment. Not actual jump cuts, but rhythmic brightness variations over the continuous shot. Medium — the stage area is framed with some crowd foreground. The strobe's ability to freeze time — each flash a purple-lit still life before time resumes in darkness. Night, intense strobe. The visual rhythm alternates between bright purple reveals and deep purple near-darkness. Electric violet (#9b0aa5) in the strobe flashes; deep purple (#2e008b) in the between-moments; soft lavender (#a082e6) persistent glow; white strobe flashes tinted purple. Rhythmic — the scene appears to stutter between frozen moments; haze moves in jerky reveals; the effect is hypnotic and dream-like, fitting the "Electric Dreams" concept.</t>
   </si>
   <si>
@@ -850,7 +854,7 @@
     <t>Mic Stand</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A chrome microphone on a stand, center stage, in the brief moment between acts or during an instrumental break. The mic and stand are surrounded by empty stage space, but the chrome surface acts as a 360-degree mirror — reflecting the colored lights, the crowd, the sky, all warped into abstract purple and violet streaks. Stage lights overhead create a pool of lavender light around the base. A thin cable snakes away into the darkness. Slow orbit around the mic stand, keeping it centered. The reflections on the chrome surface shift continuously with the orbit. Detail — the mic and the top 30cm of the stand are sharp; the stage floor and background are soft. The mic stand as a reflective sculpture — a mirror that concentrates and distorts the entire concert environment into abstract purple streaks. Night — the stage is lit from above and from the sides. The mic stand is the lone sentinel in a pool of light. Chrome reflects every color but predominantly electric violet (#9b0aa5) and soft lavender (#a082e6); deep purple (#2e008b) stage floor; pink (#eb5adc) reflected from side lights; the mic grille is dark with subtle metallic purple highlights. Slow orbit creating shifting reflections; the mic cable sways slightly from a breeze; light reflections on the chrome surface are liquid and ever-changing.</t>
   </si>
   <si>
@@ -863,7 +867,7 @@
     <t>Wristband Glow</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Hundreds of LED wristbands on raised wrists pulse in perfect unison — all electric violet, then all soft lavender, then all pink, creating waves of color that roll across the crowd. The camera tracks close above the sea of wrists, seeing each wristband as a glowing node in a larger connected network. Occasional glowing phone screens punctuate the wristband field. The wrists and arms are anonymous silhouettes connecting dark body mass to glowing band. Close tracking above the crowd, skimming over the sea of raised wristbands, moving from back of crowd toward the stage. Detail — nearest wristbands are sharp, showing their texture and glow; distant ones become a field of bokeh light points. The wristbands as collective pixels — individual nodes forming a unified, synchronized display of Electric Purple. Night — the wristbands and stage provide the only illumination. The crowd is a dark mass animated by hundreds of purple light points. Electric violet (#9b0aa5) primary wristband color; pink (#eb5adc) and soft lavender (#a082e6) in the color transitions; deep purple (#2e008b) in the spaces between lights; light blue (#7da0eb) from phone screens. Wristbands pulse in waves; the camera tracks forward; arms sway; the synchronized color changes ripple through the crowd like a digital aurora.</t>
   </si>
   <si>
@@ -879,7 +883,7 @@
     <t>Roller Coaster Lights</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A roller coaster track outlined in LED strip lights — electric violet on the rails, pink on the support structure. The camera tracks alongside at rail level as a coaster train rushes past, its own lights a streak of lavender. The track twists and curves ahead, its illuminated path drawing glowing purple lines against the night sky. Below, the park's lights are a distant carpet of warm color. Tracking alongside the coaster track at rail level, matching the train's speed for a beat, then letting it pull ahead. Wide — the track structure and its LED outlines fill the frame with geometric purple light paths. The roller coaster track as a drawn line of light — architecture becoming pure energy and movement. Night, motion. The speed of the coaster creates motion blur on the surroundings while the track LEDs stay sharp. Electric violet (#9b0aa5) LED rails; pink (#eb5adc) support structure LEDs; soft lavender (#a082e6) coaster lights; deep purple (#2e008b) night sky; electric blue (#3750dc) motion-blur of distant lights. The coaster train rushes through frame; the tracking creates a dynamic perspective; the LED lights streak at the edges; the track curves reveal new angles of light.</t>
   </si>
   <si>
@@ -895,7 +899,7 @@
     <t>Sound Wave</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 An abstract, semi-real visualization of sound waves propagating through the concert atmosphere. Concentric rings of energy expand outward from the stage in the Electric Purple palette — each ring a different shade. The waves interact with the haze, creating visible interference patterns. Where the waves pass through the crowd, wristbands pulse. Where they hit surfaces, they create ripple reflections. The scene sits between photorealism and artistic interpretation. Abstract visualization — the camera is static, but the scene itself is a dynamic wave animation overlaid on the real concert environment. Abstract — the sound waves are sharp geometric elements; the real environment beneath is slightly soft and dreamlike. Sound made visible — the invisible energy of music rendered as expanding purple light waves. Night, ethereal. This is a heightened, almost hallucinatory version of the concert — the way music feels, not just how it looks. Each concentric ring a different shade — deep purple (#2e008b) innermost, electric violet (#9b0aa5) mid-range, soft lavender (#a082e6) outer, pink (#eb5adc) furthest; electric blue (#3750dc) interference nodes. Concentric waves expanding rhythmically from the stage; interference patterns forming and dissolving; wristbands activating as waves pass; the entire scene pulses with visible sonic energy.</t>
   </si>
   <si>
@@ -917,7 +921,7 @@
     <t>Stage Fog</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Low-angle shot from the stage floor level, looking across the stage surface. Dense, heavy fog — cooled to stay low — rolls across the stage like a slow-motion purple tide. Stage lights from above pierce the fog in vertical shafts of violet and lavender. The fog's surface is not flat but turbulent, with curls and eddies catching different colored lights. In the background, the silhouette of a microphone stand rises above the fog layer like a reed above a lake. Low-angle — the lens is at fog-surface level, looking across the rolling mist. Slow forward push. Medium — the fog surface texture in the foreground is sharp; the background elements rise out of it in soft focus. The fog as a living entity — a purple sea rolling across the stage, transforming a flat surface into a landscape. Night, heavy low fog. The fog creates its own microclimate on stage — the world above the fog and below it are completely different. Soft lavender (#a082e6) and electric violet (#9b0aa5) in the fog's lit surfaces; deep purple (#2e008b) in the fog's shadows and underside; pink (#eb5adc) light shafts from above; dark silhouettes emerging from the mist. Fog rolls forward in slow, heavy waves; light shafts cut through and create shifting patterns; eddies form and dissolve; the fog reacts to unseen air currents.</t>
   </si>
   <si>
@@ -936,7 +940,7 @@
     <t>Ticket Stub</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Extreme close-up of a concert ticket held between fingers (anonymous, no identifiable features). The ticket features typographic details in purple and violet ink. The camera focuses on the paper texture — visible fibers catching the light — while the concert venue behind the ticket is a gorgeous field of purple bokeh circles of varying sizes. The ticket's edge is slightly torn where it was separated from the stub. A faint holographic security strip catches violet light. Macro static — the ticket is pinned in space; the bokeh background shifts subtly as the hand holding it sways slightly. Extreme detail — paper fibers and ink edges are sharp; the background is pure creamy bokeh. The ticket as artifact — a physical token of the experience, rendered with the intimacy of macro photography. Night — the ticket is lit by ambient stage light spillage; the background is the out-of-focus concert in full purple intensity. Purple and violet ink on white paper; deep purple (#2e008b) bokeh background; electric violet (#9b0aa5) and pink (#eb5adc) bokeh circles; soft lavender (#a082e6) holographic strip reflections. Very subtle — the hand holding the ticket sways marginally; the bokeh circles drift and shift; the holographic strip flashes as the angle changes.</t>
   </si>
   <si>
@@ -952,7 +956,7 @@
     <t>Balloons over Strandvägen</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A cluster of purple, violet, and lavender balloons ascends into the night sky above Gröna Lund. The camera tilts up to follow their flight. The balloons are backlit by the park's lights below, giving their undersides a warm glow while their tops are silhouetted against the deep purple sky. As they rise above the park's treeline, the grand Strandvägen boulevard comes into view across the harbor — its row of Art Nouveau and Jugendstil apartment buildings lit in warm amber, the historic wooden boats (Strandvägen's skärgårdsbåtar) moored along the quay, and the avenue's double row of linden trees. The balloons float between the worlds of Djurgården's park magic and Strandvägen's urban elegance. Slow tilt up — following the balloons' ascent, revealing the Strandvägen skyline as the angle widens. Wide — balloons are sharp against the sky; Strandvägen's lit facades and the park below soften into a warm light carpet. The balloons as vehicles of escape drifting from Djurgården's playground energy toward Strandvägen's sophisticated glow — two iconic Stockholm faces united in the purple night. Night, whimsical. A moment of childlike wonder with Stockholm's most elegant boulevard as backdrop. Balloons in deep purple (#2e008b), electric violet (#9b0aa5), soft lavender (#a082e6), and pink (#eb5adc); Strandvägen facades in warm amber; the sky is deep indigo; electric blue (#3750dc) harbor water between Djurgården and the boulevard. Balloons rise and slowly separate; they rotate and catch light differently; the tilt reveals Strandvägen progressively; harbor reflections connect the two shores.</t>
   </si>
   <si>
@@ -968,7 +972,7 @@
     <t>Mixing Desk</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A professional audio mixing console in the sound booth, its surface alive with color. Rows of faders, knobs, and illuminated VU meters create a landscape of precision and light. The faders are lit from below by built-in LEDs; the VU meters glow amber and green; the entire console is bathed in ambient purple light from the stage. The fader positions reflect the current mix — different heights forming a visual rhythm. Out-of-focus stage is visible in the far background through the booth opening. Slow pan across the console surface, right to left, at a low angle that emphasizes the fader heights. Detail — the nearest faders and meters are sharp; the console stretches into soft-focus distance. The mixing desk as the unseen conductor of the concert experience — every sound heard by the crowd shaped by these controls. Night, intimate. This is the backstage brain of the show, lit by its own functional lights and the ambient purple spill. Amber and green VU meters against electric violet (#9b0aa5) ambient light; deep purple (#2e008b) shadows between channels; soft lavender (#a082e6) light from the console's own illumination; fader caps catching pink (#eb5adc) stage reflections. Slow pan; faders occasionally move (ghost-operated by unseen hands); VU meters bounce with the music; LED indicators blink; the stage in the background pulses with distant purple light.</t>
   </si>
   <si>
@@ -984,7 +988,7 @@
     <t>Södermalm Waterfront View</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Ultra-wide shot from across the harbor water on the Södermalm side, framing Gröna Lund's main stage as a purple beacon on the Djurgården waterfront. The camera position near Fotografiska (Stockholm's renowned photography museum) places its distinctive red-brick industrial building at the left frame edge. The stage lights are reflected in the harbor water in long, shimmering purple and violet streaks that stretch toward the camera. The Södermalm cliff face (Stigberget) rises to the right of frame, its rooftop bars and apartments glowing warm against the purple night. Between Södermalm and Djurgården, the dark harbor water becomes a canvas of reflected purple light. Stockholm's cityscape bridges the two shores. Wide establishing — static or with an almost imperceptible slow zoom-in over 8 seconds. Ultra-wide — everything from Fotografiska's brick facade through the harbor reflections to the distant Gröna Lund stage is in focus. The concert as seen from Stockholm's cultural south bank — the stage's purple energy radiating across the water to Södermalm's creative waterfront, with Fotografiska as the cultural anchor. Night with reflections. The harbor connects Djurgården's concert energy to Södermalm's urban culture, the water multiplying the purple light. Electric violet (#9b0aa5) stage and its water reflection; deep purple (#2e008b) sky and dark water; warm red-brick of Fotografiska; soft lavender (#a082e6) in the harbor reflections; Södermalm's cliff-top lights in warm amber; pink (#eb5adc) accent lights reflected. Water choppy with shifting reflections; distant stage lights pulse; a Djurgården ferry crosses the harbor; Södermalm's cliff-top restaurants glow steadily.</t>
   </si>
   <si>
@@ -1003,7 +1007,7 @@
     <t>Encore Flash</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The encore moment — the stage erupts with a massive burst of violet and pink pyrotechnics. Geysers of purple sparks shoot upward from the stage edges. The camera rapidly zooms out to capture the full scale of the pyrotechnic display against the night sky. The sparks arc and fall in glowing parabolas, trailing lavender smoke. The crowd erupts into a sea of raised hands and phone lights. The ferris wheel in the background is dwarfed by the stage's firework display. Fast zoom out — starting close on the first spark eruption, pulling back rapidly to reveal the full spectacular display. Wide — the pyrotechnics fill the frame at multiple depths. The explosive power of the finale — contained violence of pyrotechnics rendered in the Electric Purple palette. Night, explosive. The air fills with smoke, sparks, and purple light. Maximum sensory overload. Electric violet (#9b0aa5) and pink (#eb5adc) pyrotechnic sparks; deep purple (#2e008b) smoke trails; soft lavender (#a082e6) in the illuminated smoke clouds; white-hot centers of each spark. Explosive — sparks arc upward and fall; smoke billows; the zoom-out creates a widening perspective; crowd surges; the entire scene is kinetic and alive.</t>
   </si>
   <si>
@@ -1022,7 +1026,7 @@
     <t>Rain on Lights</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A light summer rain falls through the concert's spotlight beams. Each raindrop becomes a momentary streak of colored light — purple, violet, pink — as it passes through different beams. The camera captures the rain as thousands of tiny light trails against the dark sky. Below, the wet surfaces of the stage equipment and crowd barriers reflect the purple lights in smeared, impressionist pools. A spotlight beam becomes a visible cone of falling illuminated rain. Static, looking upward at about 45 degrees into the rain and spotlights. The rain falls toward and past the camera. Detail — some raindrops are frozen sharp; others are long streaks depending on their distance from the lens. Rain as a natural light-catching medium — each drop a brief carrier of the Electric Purple palette. Night, light summer rain. The rain adds a layer of magic to the concert, not dampening the energy but enhancing the light effects. Electric violet (#9b0aa5) raindrop streaks through the main beams; deep purple (#2e008b) sky; pink (#eb5adc) drops through accent lights; soft lavender (#a082e6) in the wet-surface reflections below. Rain falls continuously in streaks of light; puddle reflections shimmer; spotlight beams become rain-shower curtains; occasional larger drops splash on surfaces.</t>
   </si>
   <si>
@@ -1041,7 +1045,7 @@
     <t>Crowd Hands</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A sea of raised hands seen from a slightly elevated angle, stretching from the foreground to the distant stage. The hands are lit from below by the stage wash, creating a field of purple-pink-lit fingers against the dark sky. Wristbands add points of glowing violet. The hands move in slow, synchronized waves — following the music's rhythm. Phone screens held aloft add bright rectangular accents. The overall effect is organic, like a field of luminous sea anemones swaying in a current. Slow tracking over the crowd — moving from above the crowd toward the stage, skimming at about 3 meters above hand height. Medium — the nearest hands are individual and detailed; further away they merge into an abstract purple-lit mass. The crowd's hands as a unified, living, luminous organism — individual gesture dissolved into collective rhythm. Night — the stage light from ahead paints the underside of every raised hand in purple and pink. Electric violet (#9b0aa5) and pink (#eb5adc) underlit skin; deep purple (#2e008b) dark sky above; soft lavender (#a082e6) wristband glow; light blue (#7da0eb) phone screens. Hands sway in slow waves; phone screens appear and disappear; wristbands pulse; the tracking creates a flowing perspective over the living sea of hands.</t>
   </si>
   <si>
@@ -1057,7 +1061,7 @@
     <t>Vinyl Spin</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A vinyl record spins on a turntable at the DJ booth side-stage. The camera captures the record at macro level — the grooves are visible as concentric lines that catch the ambient purple stage light in shifting patterns. The record label at the center is a design in Electric Purple tones. The tonearm sits in the groove, its cartridge reflecting a tiny version of the stage lights. Warm amber light from the DJ booth's equipment contrasts with the purple ambient. Macro orbit — slowly circling the spinning record, keeping the groove detail in focus as the reflections shift. Detail — the grooves and their light reflections are the subject; the DJ booth and stage beyond are soft purple bokeh. The vinyl record as both musical medium and optical surface — its grooves a physical encoding of sound that also reflects the visual spectacle. Night, with a retro warmth. The turntable setup evokes analog craft in a digital world. Black vinyl catching electric violet (#9b0aa5) and soft lavender (#a082e6) reflections in the grooves; deep purple (#2e008b) in the record's shadowed areas; pink (#eb5adc) label; warm amber from the booth lights. The record spins at 33rpm — the grooves create concentric moving reflections; the orbit adds a second layer of shifting perspective; the tonearm vibrates microscopically; light patterns on the vinyl surface are hypnotic.</t>
   </si>
   <si>
@@ -1076,7 +1080,7 @@
     <t>Final Beam over Djurgården</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The concert's final moment. All stage lights — which have been a complex symphony of colors — slowly converge into a single, vertical beam of pure electric violet rising from Gröna Lund's stage into the Stockholm sky. The haze catches this beam beautifully, making it a solid column of purple light visible across the city. As the camera slowly dollies back across the harbor, the beam becomes a landmark visible in context with Stockholm's skyline — Stadshuset's tower to the left, Gamla Stan's spires to the right, and the purple beam from Djurgården standing between them as a temporary fourth spire of Stockholm. The crowd watches in silence. Then, gently, the beam fades to black, and only the permanent city lights remain. Slow dolly back across the harbor — pulling away from Djurgården, contextualizing the beam within Stockholm's wider skyline. Wide — the beam is a singular vertical element among Stockholm's silhouetted landmarks. The purple beam as a temporary addition to Stockholm's skyline — standing alongside Stadshuset and Gamla Stan's spires, then vanishing, leaving only the memory of Electric Purple. Night, closing. The energy shifts from chaos to order to silence. The beam connects Djurgården to the sky for one final moment. Pure electric violet (#9b0aa5) in the beam; deep purple (#2e008b) sky; warm amber on Stadshuset and Gamla Stan; soft lavender (#a082e6) scattered by the haze; as the beam fades, the city's warm tones gradually dominate and the purple drains to dark (#34303d). Slow dolly back; the beam stands still among Stockholm's landmarks; haze drifts through it; the beam slowly dims; the city lights persist as the purple fades.</t>
   </si>
   <si>
@@ -1101,7 +1105,7 @@
     <t>Steam Rise</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Inside a dimly lit sauna. Dense white-gray steam rises from a pile of dark hot stones, billowing upward in slow, organic plumes. A light source above — unseen, but casting deep purple and violet — illuminates the steam from behind, turning each plume into a column of glowing lavender and violet. The dark wooden walls of the sauna absorb most light, creating a cave-like intimacy. The stones at the base glow a deep amber-red between their gaps. Slow tilt up — starting on the glowing stones, rising through the steam plumes toward the purple light source above over 8 seconds. Medium — the steam is the mid-ground subject; the stones below are warm and slightly soft; the ceiling above is lost in purple-lit mist. Steam as the medium for light — transforming invisible water vapor into a visible, purple-lit sculpture. Warm interior, dim. The heat is palpable. The air is thick with moisture. The only lights are the stone glow and the purple ambient above. Deep amber-red on the stones; electric violet (#9b0aa5) and soft lavender (#a082e6) in the backlit steam; deep purple (#2e008b) in the wooden walls and shadows; pink (#eb5adc) where the hot and cool light mix in the steam. Steam rises in slow, billowing plumes that curl and fold; the tilt follows the steam's upward journey; the stone glow pulses very gently with residual heat.</t>
   </si>
   <si>
@@ -1117,7 +1121,7 @@
     <t>Cold Plunge Entry</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The surface of a cold plunge pool — dark, still, purple-tinted water — is broken by an entry. In ultra slow motion, the water surface depresses, then erupts into a crown of droplets. Each droplet catches the dawn light in purple, lavender, and cold blue. Beneath the surface, a cloud of silver bubbles expands. The water's surface tension creates a temporary membrane before yielding. The surrounding wooden pool edge frames the shot. Slow-motion downward — capturing the entry and splash from a 45-degree angle above. Detail — the splash crown is sharp; individual droplets are frozen; the water's depth is soft purple. The moment of immersion — the shock of cold water captured as a beautiful, violent event in purple light. Dawn, cold blue. The early morning light is cold and purple, with no warmth yet. The water temperature is near-freezing — the visual language should feel cold. Deep purple (#2e008b) in the undisturbed water; electric blue (#3750dc) and light blue (#7da0eb) in the cold splash highlights; soft lavender (#a082e6) in the frozen droplets; silver-white in the bubbles; warm wood tones at the frame edges. Ultra-slow-motion splash: water depression, crown formation, droplet separation, bubble cloud expansion. The violence of the entry rendered as slow, beautiful physics.</t>
   </si>
   <si>
@@ -1136,7 +1140,7 @@
     <t>Wooden Grain</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Extreme macro of cedar wood — the sauna's bench surface. The wood grain is a landscape of ridges and valleys, its growth rings telling decades of story. Warm amber light from one direction catches the grain ridges while purple-tinted shadow fills the valleys. The wood has the slight sheen of heat and moisture. Tiny droplets of condensation sit in the grain channels like rivers on a topographic map. A single knot in the wood is a dark eye in the amber field. Macro drift — slowly panning across the wood surface, as if exploring a terrain from above. Extreme detail — individual wood fibers and condensation droplets are visible. The drift takes the focus through different depth planes. The cedar wood as a micro-landscape — nature's pattern language rendered visible by the interplay of warm and purple light. Warm, intimate. The macro perspective transforms the familiar sauna bench into an alien, beautiful terrain. Warm amber and honey on the grain ridges; deep purple (#2e008b) in the grain valleys; electric violet (#9b0aa5) in the deeper shadows; soft lavender (#a082e6) on the condensation droplets catching reflected sky through a window. Slow lateral drift across the wood surface; condensation droplets merge and slide imperceptibly; a rising heat distortion softens the far edge of the macro view.</t>
   </si>
   <si>
@@ -1152,7 +1156,7 @@
     <t>Riddarfjärden Float</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A wooden sauna structure — a minimalist Nordic box with warm light spilling from its windows — floats on the waters of Riddarfjärden, the iconic body of water at the heart of Stockholm. The distinctive silhouette of Stadshuset (Stockholm City Hall) with its tower and three golden crowns is visible on the northern shore, its red-brick facade catching the last ambient light. To the east, the profile of Gamla Stan's rooftops and church spires rises against the purple sky. The Riddarfjärden surface is a flawless mirror of the blue-hour sky, making the sauna appear to hover between the reflected city and the real one. A thin layer of mist floats just above the water, catching the sauna's window glow in soft amber wisps. Slow orbit — the camera circles the floating sauna roughly 20 degrees over 8 seconds, shifting the backdrop from Stadshuset to Gamla Stan. Wide — the sauna, its reflection, the mist layer, and Stockholm's landmark silhouettes are all in focus. The floating sauna centered in Riddarfjärden — the ultimate Stockholm wellness fantasy, bathing with the city's most iconic landmarks as your backdrop. Blue hour with low mist on Riddarfjärden. The scene is hushed and meditative despite the urban setting. The city feels distant, dream-like. Warm amber from the sauna windows; deep purple (#2e008b) sky and its water mirror; Stadshuset's red brick in muted warm tones; electric violet (#9b0aa5) at the horizon; soft lavender (#a082e6) mist catching the window glow; Gamla Stan as a warm amber cluster. Slow orbit; the reflected city shifts with the camera; mist drifts lazily; window glow flickers (fire inside); the sauna bobs imperceptibly; Stadshuset's tower light glows steadily.</t>
   </si>
   <si>
@@ -1165,7 +1169,7 @@
     <t>Hot Stones</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The löyly ritual — water is poured from a wooden ladle onto searing hot sauna stones. The moment of contact produces an explosive release of steam — a violent, beautiful eruption that fills the frame. The stones themselves glow deep amber-red in their crevices. The steam shoots upward and outward, instantly catching purple light from above. Water droplets that don't immediately evaporate dance and skitter across the stone surface like tiny mercury balls. Static, positioned at stone level, facing the pour point directly. The steam eruption fills the frame. Detail — the stone surfaces and the point of water contact are sharp; the steam explosion above is volumetric and slightly soft. The moment of transformation — liquid water becoming steam on contact, a phase change rendered as visual spectacle. Warm interior — the heat is at its peak during the löyly. The air is already saturated with moisture; this pour pushes it further. Deep amber-red on the hot stones; white-to-lavender (#a082e6) steam; deep purple (#2e008b) in the dark sauna interior beyond; electric violet (#9b0aa5) in the backlit upper steam; dancing water droplets catch pink (#eb5adc) light. Water stream contacts stones; explosive steam eruption; skittering water droplets; the steam plume rises and expands; the ladle tilts (seen at frame edge) controlling the pour.</t>
   </si>
   <si>
@@ -1184,7 +1188,7 @@
     <t>Breath Cloud</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Close-up of a visible breath cloud — a warm exhalation in freezing air. The breath is backlit by the purple dawn light, turning it into a slow-motion sculpture of swirling vapor. Each exhale creates a new shape: first a compact jet, then it blooms and unfolds, curling at the edges before dissipating into the purple air. The anonymous subject is barely visible — just the silhouette of a chin and lips at the very bottom of frame. The background is a purple gradient dawn sky. Slow-motion, fixed on the breath zone. Multiple exhales are captured in the 8 seconds, each creating and destroying a new vapor sculpture. Detail — the breath vapor is sharp in the center of its cloud; the edges dissolve into the purple air. Breath as visible proof of the body's heat meeting the cold outside — the primal contrast of the sauna experience. Cold exterior, dawn. The temperature contrast between the warm body (just out of the sauna) and the freezing morning air is extreme. White and soft lavender (#a082e6) in the breath vapor; electric violet (#9b0aa5) backlight glow through the vapor; deep purple (#2e008b) background sky; pink (#eb5adc) at the edges where vapor meets purple light. Slow-motion breath clouds: ejection, bloom, curl, dissipation. Each breath is unique. The vapor interacts with any ambient air movement, creating unpredictable, beautiful shapes.</t>
   </si>
   <si>
@@ -1200,7 +1204,7 @@
     <t>Brunnsviken Mirror</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A perfectly symmetrical composition on the waters of Brunnsviken — the serene lake north of Stockholm's center, bordered by the royal Haga Park. The frame is divided exactly at the waterline. Above: the floating sauna with its warm-lit windows, the dark silhouette of Haga Park's ancient oaks and the distinctive copper roof of the Haga Palace pavilion visible on the far shore, and the deep purple-violet blue-hour sky. Below: a flawless mirror reflection of everything above, slightly darker and more purple. The famous Haga Park lawns slope gently to the waterline behind the sauna. Brunnsviken's sheltered waters are perfectly still. Low-angle wide — the lens is at exact waterline level, creating the symmetrical split. Static or with an imperceptible forward float. Ultra-wide — sharp from the nearest water surface to Haga Park's tree line. The symmetry demands total clarity. Brunnsviken as Stockholm's most tranquil body of water — the sauna floating in the royal park's mirror lake, suspended between two reflected purple worlds. Blue hour, dead calm. Not a breath of wind on Brunnsviken's sheltered surface. The royal park creates a buffer of silence from the city. Deep purple (#2e008b) sky and its deeper reflection; electric violet (#9b0aa5) at both horizons; soft lavender (#a082e6) in the lighter sky; warm amber from the sauna windows doubled by the reflection; Haga Park's dark greens reading as deep purple in the evening light. Near-static — the only movement is a very slight bob of the sauna and an occasional micro-ripple from a diving bird that momentarily distorts the perfect Haga Park reflection.</t>
   </si>
   <si>
@@ -1216,7 +1220,7 @@
     <t>Ice Crystals</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Extreme macro of ice crystals formed on the sauna's exterior window. The crystals are intricate fractal patterns — fern-like dendrites and hexagonal plates — each catching the ambient purple light at different angles. Through the ice, the warm amber interior of the sauna is visible but distorted into abstract blobs of warm color. The ice itself is a spectrum of clear, white, and pale blue, with the purple light turning it into a natural stained-glass window. Macro — static or with an impossibly slow drift across the ice surface, revealing new crystal formations. Extreme detail — individual ice crystal branches are sharp; the warm interior beyond is bokeh. Ice crystals as nature's fractal art — the cold's beautiful answer to the heat within. The contrast between frozen surface and warm interior is the sauna's essence. Cold, crystalline. The ice exists because the interior is warm and the exterior is freezing — each crystal is evidence of the temperature gradient. Clear and pale blue ice; electric violet (#9b0aa5) and soft lavender (#a082e6) light caught in crystal facets; deep purple (#2e008b) in the shadows between crystals; warm amber bokeh from the interior beyond; occasional pink (#eb5adc) refraction through the crystal prisms. Extremely slow drift across the crystal landscape; occasional crystal glint as the angle shifts; the warm interior beyond the ice shimmers softly; a very slow melt — a tiny water bead forming and beginning to run.</t>
   </si>
   <si>
@@ -1235,7 +1239,7 @@
     <t>Ember Glow</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Close-up of the sauna stove's ember bed. Charcoal and wood pieces glow in deep amber, orange, and red — a miniature volcanic landscape. The embers pulse with residual heat, brightening and dimming in slow breathing cycles. Above the ember bed, heat distortion warps the view of the dark sauna interior. The stones above the embers are dark but their undersides catch a deep purple-red glow. Tiny sparks occasionally float upward from the ember surface. Static — locked on the ember bed. The stillness allows the viewer to become mesmerized by the slow pulsing of the embers. Detail — the ember surfaces are sharp, showing cracked charcoal texture and glowing fissures; the area above shimmers with heat distortion. The ember bed as the heart of the sauna — its steady glow is the source of all warmth, all steam, all ritual. Warm interior, dim. The ember glow is the primary light source in this shot, casting everything in its amber-red-purple spectrum. Deep amber and red in the ember cores; the outer charcoal surfaces shift to deep purple (#2e008b) and electric violet (#9b0aa5); the stones above catch soft lavender (#a082e6) from the mixed ember-and-ambient light; the heat distortion above carries pink (#eb5adc) shifts. Embers pulse slowly (brightening over 2 seconds, dimming over 3); occasional tiny sparks drift upward; heat distortion shimmers above the bed; a piece of charcoal shifts and settles, releasing a brief burst of new glow.</t>
   </si>
   <si>
@@ -1248,7 +1252,7 @@
     <t>Långholmen Mist</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A thin layer of mist — only about half a meter thick — hovers over the water surface near Långholmen island at dawn. This is one of Stockholm's most beloved urban nature spots — the former prison island turned into a green oasis in the city's heart. The camera glides through the mist layer at water level, pushing through it like moving through a violet cloud. Through breaks in the mist, the Långholmen shoreline is visible — its distinctive yellow cliffside former prison buildings, now a hotel and hostel, rising above the trees. The Västerbron bridge arches across the sky in the background, its span catching the first purple-gold light. Above the mist, Långholmen's dense deciduous canopy is a dark mass against the purple sky. Slow dolly forward through the mist layer at water level, approaching Långholmen from the Riddarfjärden side. Wide — the mist has depth; Långholmen's shore reveals itself through the mist; Västerbron frames the background. The mist as a veil between the urban waterway and the hidden natural paradise of Långholmen — the city's most surprising green island emerging from a purple cloud. Dawn, misty. Stockholm is still asleep. The mist transforms a familiar urban waterway into a dreamscape where Långholmen feels like a hidden island in a fairy tale. Soft lavender (#a082e6) and white in the illuminated mist; deep purple (#2e008b) water below and sky above; electric violet (#9b0aa5) where the mist is backlit by the brightening horizon behind Västerbron; the yellow Långholmen buildings add warm amber accents. Forward glide through the mist toward Långholmen; mist parts and closes; Västerbron's silhouette grows clearer; occasional clear patches reveal the dark water below; birdsong is implied by a heron silhouette taking flight from the shore.</t>
   </si>
   <si>
@@ -1264,7 +1268,7 @@
     <t>Water Droplets</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Extreme macro of water droplets condensing and running down the warm wooden interior wall of the sauna. Each droplet is a perfect lens, refracting and inverting the warm amber interior light. The droplets merge, grow heavy, and begin to slide, leaving wet trails on the wood. The wood grain is visible through and around the droplets. A faint purple ambient light from the window mixes with the warm interior, creating a dual-tone illumination. Macro slow-motion — fixed on a section of wall, capturing the slow life cycle of condensation droplets. Extreme detail — individual droplets are large enough to see refracted images within them. The wood grain texture is fully resolved. Condensation as evidence of heat — the warm, moist air of the sauna manifested as jewel-like droplets on wood. Warm interior — the high humidity is visible in the condensation. The air itself feels thick and warm. Warm amber refracted through the droplets; the wet wood is darker, revealing deep purple (#2e008b) in its grain; soft lavender (#a082e6) from the window light catching individual droplets; the dry wood is warm honey-tone. Droplets form, grow, merge, and begin to slide in ultra-slow-motion; each sliding droplet leaves a wet trail that darkens the wood; new droplets form in the trail; the process is meditative and endless.</t>
   </si>
   <si>
@@ -1280,7 +1284,7 @@
     <t>Plunge Bubbles</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Underwater perspective looking upward in the cold plunge pool. A cloud of silver-white air bubbles rises toward the surface, each bubble a tiny spherical mirror reflecting the purple world above. The water is tinted deep purple-blue by the sky light filtering through the surface. The surface itself is a shimmering, distorted window — the purple sky and sauna structure visible but wavering above. Sunbeams (or pre-dawn light beams) penetrate the water in shafts of electric violet. Underwater, looking up at about 30 degrees. Static, allowing the bubbles to rise through and past the frame. Detail — the nearest bubbles are sharp enough to see reflections in them; distant bubbles and the surface are soft and dreamy. The bubbles as ascending spheres of captured breath — each one a tiny reflection of the world above, rising from the cold depths. Cold, underwater. The world below the surface is silent, slow, and deeply purple. A meditative counterpoint to the violent splash of entry. Deep purple (#2e008b) and electric blue (#3750dc) in the water body; soft lavender (#a082e6) and electric violet (#9b0aa5) in the light shafts; silver-white bubbles with purple reflections; the surface above is a luminous purple-gold window. Bubbles rise in slow, wobbly ascent; they merge when they touch, forming larger bubbles that accelerate; light beams shift as the surface undulates; the overall feeling is peaceful and ascending.</t>
   </si>
   <si>
@@ -1299,7 +1303,7 @@
     <t>Smoke Curl</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A single, elegant curl of steam or smoke rises from the sauna's stone pile, illuminated by a narrow beam of purple light against a completely dark background. The curl follows a complex, organic spiral — twisting, folding back on itself, branching — creating a temporary natural sculpture. The beam catches the smoke/steam at different densities — thick sections glow brightly, thin sections are translucent ghosts. The dark background is not true black but deep indigo-purple. Static — the smoke curl is the performance; the camera is the audience. Centered composition. Detail — the smoke edges are sharp where dense, dissolving to nothing where thin. The background is a uniform deep purple. The smoke curl as calligraphy — a natural brushstroke of steam writing in purple light against darkness. Wabi-sabi in motion. Dim, atmospheric. This is a meditative moment — a single element in near-darkness. The sauna stripped to its essence. White-to-lavender (#a082e6) in the dense smoke; electric violet (#9b0aa5) at the beam edges; deep purple (#2e008b) background; occasional pink (#eb5adc) where the thinnest wisps catch the light at oblique angles. The smoke curl rises and evolves continuously — no two frames are alike. It twists, folds, blooms, and dissipates in a perpetual, unrepeatable dance.</t>
   </si>
   <si>
@@ -1315,7 +1319,7 @@
     <t>Birch Whisk</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A traditional Finnish birch whisk (vihta) swings through the steamy sauna air in slow motion. The bundle of birch branches with their small green leaves cuts through the steam, creating swirling vortices in its wake. Water droplets fly off the leaves in a spray pattern. The leaves are backlit by the purple-amber sauna light, making them glow translucent green with purple edges. Steam parts and reforms around the whisk's path. Slow-motion swing — the camera tracks the whisk through its arc, positioned to catch the backlit leaf spray and steam vortices. Detail — the whisk bundle and its immediate spray zone are sharp; the steam-filled background is soft purple. The vihta as a traditional tool of ritual — birch leaves and steam and heat combined in an ancient Nordic practice. Warm interior — the sauna is at full heat. Steam is dense. The whisk ritual is the peak of the sauna experience. Translucent green leaves backlit with amber and electric violet (#9b0aa5); water droplets catching purple and pink (#eb5adc) light; deep purple (#2e008b) in the background steam; soft lavender (#a082e6) in the nearest steam wisps. The whisk swings in a slow arc; leaves flutter; water droplets spray in a fan pattern; steam vortices spiral in the whisk's wake; everything is slow-motion ballet.</t>
   </si>
   <si>
@@ -1331,7 +1335,7 @@
     <t>Hellasgården Frozen Pier</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A frost-covered wooden pier extends from the shore of Hellasgården — Stockholm's beloved outdoor recreation area on the shores of Lake Källtorp in the Nacka nature reserve. This is where Stockholmers have practiced traditional Nordic wellness for generations — sauna, ice swimming, forest bathing. Every surface of the pier is coated in white frost crystals that catch the pre-dawn purple light. The familiar Hellasgården sauna buildings with their characteristic red wooden walls are visible on shore. At the pier's end, a floating sauna structure glows amber from within. The frozen lake surface stretches toward forested hills — Nacka's nature reserve is a wall of dark purple-green. The dawn sky is a deep gradient from indigo to electric violet. Slow dolly forward along the Hellasgården pier, creating a sense of approach toward the warm sauna — the iconic walk every winter bather knows. Wide — the frosted pier details in the foreground; the familiar red Hellasgården buildings on shore; the sauna and dawn sky ahead. The Hellasgården pier as a pilgrimage path — every Stockholmer recognizes this walk from shore to sauna as the ritual beginning of the Nordic bathing experience. Winter dawn at Hellasgården — bitterly cold. The frost is thick. The Nacka forest stands as a dark guardian around the frozen lake. White frost with lavender (#a082e6) and electric violet (#9b0aa5) tints; deep purple (#2e008b) sky and frozen lake; Hellasgården's red buildings as warm contrast; warm amber from the sauna windows ahead; the Nacka forest is deep purple-green. Slow forward dolly; frost crystals catch and release light; the sauna's warm glow grows; the familiar red buildings pass at the frame edge; breath-like mist drifts at the pier surface.</t>
   </si>
   <si>
@@ -1350,7 +1354,7 @@
     <t>Thermometer Rise</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A traditional wooden sauna thermometer/hygrometer mounted on the wall. The camera captures the temperature dial at macro level as the reading climbs — the needle sweeping from the comfortable zone into the high-heat zone. The dial face is marked in vintage typography. The wooden housing catches warm amber light from the sauna's stove while purple light from outside the window creates a cool accent on the glass surface. Condensation beads form on the glass face. Macro time-lapse feel — the needle's movement is the drama, everything else is near-static. Detail — the needle and dial markings are crisp; the wooden housing frame softens at the edges. The thermometer as the objective witness to the sauna's rising heat — a scientific instrument in a sensorial environment. Warm, building. The temperature is climbing. The sauna is being prepared — the ritual has not yet begun but the conditions are being set. Warm amber on the wooden housing; the dial face reflects both amber (stove) and electric violet (#9b0aa5) (window); the needle is dark against deep purple (#2e008b) dial markings; soft lavender (#a082e6) condensation droplets on the glass. The needle sweeps slowly upward; condensation droplets form and grow on the glass; the warm-cool light balance shifts as the stove builds heat; a subtle vibration from the heating wood structure.</t>
   </si>
   <si>
@@ -1369,7 +1373,7 @@
     <t>Ripple Ring</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Looking straight down at a perfectly still lake surface. A single water drop falls and strikes the surface, creating a set of concentric ripple rings that expand outward in a perfect circle. The water reflects the purple sky, so each ripple ring is a moving circle of light and dark purple. The ripples interact with the reflected image of the floating sauna, momentarily distorting its warm window glow into shimmering fragments. As the ripples reach the frame edge, the water returns to stillness. Overhead — looking straight down at the water surface. Static. The geometry of the expanding circles is the entire composition. Detail — the ripple edges are sharp; the reflected scene in the water is visible but secondary to the wave pattern. The single ripple as a metaphor for the sauna experience — one action (a drop, a breath, a choice) creating expanding circles of effect. Still, meditative. The world is so quiet that a single drop creates a visible event. Ultimate Nordic calm. Deep purple (#2e008b) in the still water; the ripple crests catch soft lavender (#a082e6) and electric violet (#9b0aa5) sky reflections; warm amber fragments where the sauna reflection is distorted; the drop impact creates a momentary white flash. The drop impact; concentric ripples expanding at decreasing speed; the reflected sauna image fragmenting and reassembling; the slow return to perfect stillness.</t>
   </si>
   <si>
@@ -1385,7 +1389,7 @@
     <t>Towel Fold</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A white linen towel falls through the air in extreme slow motion, caught in a cross-light of warm amber from one side and electric violet from the other. The fabric billows, folds, and ripples as air catches it — each fold creating complex shadows in purple while the surfaces facing the warm light glow amber-white. The towel slowly settles onto a wooden bench, its folds recording the motion of its fall. The linen's weave texture is visible at the macro level. Slow-motion drape — tracking the towel's descent from a 45-degree angle, close enough to see the fabric texture. Detail — the nearest fabric folds are razor-sharp; the falling motion creates soft areas where the fabric is in between positions. The white linen as a surface for the dual light — warm and purple — and as a symbol of the sauna's simplicity and purity. Warm, soft. The moment after the sauna session — clean, calm, cared-for. White linen with warm amber highlights and electric violet (#9b0aa5) shadows in the folds; the wooden bench below is deep amber with purple (#2e008b) in its grain; soft lavender (#a082e6) where the two light sources mix on the fabric; the falling motion blur has a pink (#eb5adc) tint. Ultra-slow-motion drape — the towel descends, billows, catches air, folds, and settles. Each fold is a unique event. The fabric's weight and texture dictate its behavior.</t>
   </si>
   <si>
@@ -1404,7 +1408,7 @@
     <t>Window Condensation</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The sauna's window is completely fogged with condensation. Through the misted glass, the purple lake and sky beyond are visible as soft, impressionist blurs of color — deep purple water, violet sky, a hint of distant island. A single streak appears as condensation begins to run, creating a clear channel through the fog. Through this channel, the outside world snaps into sharp, vivid purple clarity — a window within a window. More streaks follow, creating abstract vertical clear paths through the fog. Static — close on the window surface. The clearing condensation is the action. Detail — the condensation droplets on the glass are in focus; the world beyond shifts between soft (through fog) and sharp (through clear streaks). The condensation as a veil between the warm interior world and the cold purple exterior — and the act of clearing it as a slow reveal. Warm interior contrasting with cold exterior. The condensation is the visible boundary between two temperature zones. The fogged glass is a neutral gray-lavender; the clear streaks reveal deep purple (#2e008b) water and electric violet (#9b0aa5) sky; soft lavender (#a082e6) in the diffused fog sections; the condensation droplets themselves catch warm amber from the interior. Condensation streaks slowly growing as gravity pulls water down; new clear channels appearing; the view through them sharpening; the purple outside world being gradually revealed in vertical stripes.</t>
   </si>
   <si>
@@ -1423,7 +1427,7 @@
     <t>Candle Row</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A row of small votive candles sits on the sauna's lower bench, their flames flickering in unison with the gentle air currents. The camera moves slowly along the row, passing each candle. Each flame is a warm amber core surrounded by a soft purple halo (from the ambient light mixing with the flame's warm tone). The candles cast dancing shadows on the wooden wall behind them — each shadow a moving silhouette that amplifies the flame's motion. The wood between the candles catches warm-cool light in alternating pools. Slow dolly along the candle row at flame height, each candle passing through focus in sequence. Detail — each candle flame is momentarily razor-sharp as the dolly passes, with the others falling to soft bokeh in both directions. The candle flames as living light sources — each one unique, all responding to the same invisible air currents, creating a rhythm of light and shadow. Warm, intimate. The candles are the only light source. The sauna is at rest — the heat session is complete, and this is the contemplative afterglow. Warm amber flame cores; soft lavender (#a082e6) halos around each flame where warm and ambient light mix; deep purple (#2e008b) in the wall shadows; the wood between candles alternates between amber highlight and electric violet (#9b0aa5) shadow. Slow dolly; each flame flickers independently but in sympathetic rhythm; shadows dance on the wall; the focus shift from candle to candle creates a breathing, rack-focus effect.</t>
   </si>
   <si>
@@ -1439,7 +1443,7 @@
     <t>Brunnsviken Ice Hole</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Bird's-eye view of frozen Brunnsviken — the beautiful lake bordered by Haga Park and the university campus. The ice is white-gray with purple shadows and frost patterns. A dark circular hole has been cut in the ice near the Haga Park shore — a perfect black circle of open water that reads as a portal to another world. Next to the hole, a floating sauna sits in its own clear-water dock. Steam rises from the sauna's chimney — a white plume against the purple environment. Footprints in the frost lead from the sauna to the ice hole. The Haga Park royal lawns and ancient oaks are visible along the eastern shore; the university buildings are a geometric pattern on the western bank. The frozen lake is framed by Stockholm's distinctive mix of nature and architecture. Overhead drone — high enough to see the sauna, ice hole, and the surrounding Brunnsviken context. Slow descent over 8 seconds. Wide — the graphic elements (dark circle, white ice, sauna rectangle, Haga Park shoreline) are all sharp in a minimalist composition. The ice hole as a dark portal in Brunnsviken's frozen surface — framed by Haga Park's royal nature, this is Stockholm's most refined setting for the primal act of ice bathing. Winter, stark. The composition is almost abstract from above — but the recognizable Haga Park context anchors it in Stockholm. White-gray ice with purple (#2e008b) shadows; the ice hole is near-black with electric violet (#9b0aa5) water reflections; soft lavender (#a082e6) in the frost patterns; warm amber from the sauna's windows; Haga Park's trees as dark purple-green; white steam against deep purple sky. Slow drone descent; the steam plume drifts; the black water in the ice hole shimmers; the descending perspective reveals Haga Park's landscape and the Brunnsviken shoreline in increasing detail.</t>
   </si>
   <si>
@@ -1458,7 +1462,7 @@
     <t>Heat Waves</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The sauna's roof ventilates heat — visible as a shimmering column of heat distortion rising from the chimney and roof surface. The camera looks through this distortion at the purple sky and distant landscape beyond, which warp and ripple like a mirage. The heat distortion acts as a living lens, bending the straight horizon line into waves. The wooden roof surface below the distortion radiates warmth — its surface slightly steaming. A bird flying in the background passes through the distortion zone and momentarily warps. Static — positioned to capture the heat distortion between the camera and the purple sky. The distortion itself is the subject. Medium — the roof edge is sharp; the heat distortion zone is the visually active area; the sky beyond is rendered surreal by the bending. Heat made visible — the sauna's invisible energy output rendered as a visual effect that transforms the purple landscape into a living painting. Warm exterior — the sauna is radiating its heat into the cold purple air. The temperature difference creates a visible optical phenomenon. The sky's electric violet (#9b0aa5) and deep purple (#2e008b) are distorted into wavy versions of themselves; soft lavender (#a082e6) in the lighter distortion zones; warm amber on the wooden roof surface; the distortion adds a pink (#eb5adc) chromatic shift at the wave edges. The heat distortion shimmers and ripples continuously; the sky and horizon warp in slow waves; steam wisps mix with the heat column; the distant bird warps as it passes through the distortion zone.</t>
   </si>
   <si>
@@ -1477,7 +1481,7 @@
     <t>Södermalm Snow Scene</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 Gentle snowfall over Riddarfjärden where the floating sauna sits, with the dramatic cliff face of Södermalm — Stockholm's creative south island — rising as a dark wall behind it. The iconic Södermalm skyline is visible along the cliff top: Monteliusvägen's viewing terraces, the distinctive rooftops of Mariaberget, and the church spire of Maria Magdalena kyrka, all softened by the falling snow. Large, slow snowflakes descend through the frame, each one catching the purple dusk light. The floating sauna is centered in the composition between the vast cliff and the open water, its warm-lit windows creating amber rectangles against the purple-gray environment. The Riddarfjärden surface is dark and still. Slow wide — static or with an almost imperceptible drift. The snowfall is the motion; Södermalm's cliff is the backdrop. Wide — the sauna is sharp at center; Södermalm's cliff face and rooftops provide dramatic scale; snowflakes vary from large and soft to tiny distant points. The floating sauna dwarfed by Södermalm's cliff — a small, warm human refuge at the base of the city's most dramatic natural feature, veiled in falling snow. Winter dusk with snowfall over Riddarfjärden. Stockholm's south cliff looms protectively. The snow muffles the city. White snowflakes with lavender (#a082e6) tint; deep purple (#2e008b) sky and Södermalm cliff shadow; electric violet (#9b0aa5) at the horizon; warm amber from the sauna windows; Södermalm's rooftop lights as tiny warm points along the cliff top. Snowflakes descend in slow, irregular paths; the sauna's chimney steam mixes with the snow; warm window glow flickers; the Södermalm cliff face catches and releases snow in patterns.</t>
   </si>
   <si>
@@ -1496,7 +1500,7 @@
     <t>Ladle Pour</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 A wooden ladle tips and water pours in a single, elegant stream onto the sauna stones below. In slow motion, the water stream catches the light — it is a glass-like cylinder that refracts the warm amber stone-glow and the purple ambient light simultaneously. Where the stream hits the first stone, it shatters into droplets and steam. The stream itself has a hypnotic quality — its surface ripples and twists as gravity pulls it downward. The ladle's wooden bowl is visible at the top of frame, its grain and patina telling years of use. Slow-motion, positioned to capture the full arc of the pour — from ladle tip to stone impact — in a vertical composition. Detail — the water stream is the sharp subject at the center; the ladle above and the stones below are slightly soft. The water stream as a liquid bridge between the wooden ladle (human intent) and the hot stones (natural element) — the ritual's central gesture. Warm interior at peak temperature. The pour is the ceremonial act that transforms heat into steam, stone into experience. The water stream refracts both amber (from stones) and electric violet (#9b0aa5) (from ambient) as internal caustics; the stone surfaces are deep amber with purple (#2e008b) shadows; the steam explosion at impact is white blooming to lavender (#a082e6); the ladle's wood is warm honey with purple grain shadows. The water stream descends in slow motion, its surface alive with tension and internal light; the impact point erupts in steam and spray; the ladle tilts imperceptibly, controlling the flow; steam rises from below.</t>
   </si>
   <si>
@@ -1509,7 +1513,7 @@
     <t>Saltsjön Dawn</t>
   </si>
   <si>
-    <t xml:space="preserve">Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
+    <t>Cinematic, dreamlike vertical video. Color palette built around "Electric Purple" — deep purples (#2e008b), electric violets (#9b0aa5), soft lavenders (#a082e6), accent pinks (#eb5adc) and electric blues (#3750dc / #7da0eb). Shadows tinted deep indigo-purple, highlights bloom into lavender and pink. Smooth slow-motion camera movements, shallow depth of field, anamorphic bokeh. Subtle lens flares, golden-hour warmth filtered through purple atmospheric haze. Strong backlight, volumetric light, filmic grain like Kodak Vision3 500T. Dreamlike, aspirational, sensorial mood. Loop-friendly motion.
 The floating sauna in silhouette against a breaking dawn sky over Saltsjön — the salt-water inlet that connects Stockholm to the Baltic Sea. The sky transitions from deep purple at the top through electric violet to a band of hot pink at the horizon where the sun is about to appear. The sauna is a dark geometric shape — a rectangle with its chimney — centered in the frame. Behind it, the familiar green silhouette of Djurgården island is visible — its oak canopy and the profile of Nordiska Museet recognizable even in silhouette. To the right, the entrance to Stockholm's inner harbor and the distant Gröna Lund ferris wheel structure are faintly visible. A faint glow of dying fire light escapes from the sauna's window — a warm amber slit in the dark form. Saltsjön's surface mirrors everything. A single bird flies from Djurgården across the purple sky. Slow dolly back — starting relatively close to the sauna, pulling away over 8 seconds to reveal the Saltsjön panorama and Stockholm's waterfront landmarks. Wide — the sauna silhouette is a graphic element; the dawn sky, Djurgården's silhouette, and Saltsjön's reflections fill the composition. The sauna on Saltsjön at dawn — where Stockholm's salt water meets the Baltic, with the city's cultural island as backdrop. The session ends as the city awakens. Dawn, clear over Saltsjön. The first light arrives from the Baltic. The sauna session is ending. A new Stockholm day begins in the Electric Purple palette. Deep purple (#2e008b) sky at top; electric violet (#9b0aa5) mid-sky; pink (#eb5adc) at the horizon; soft lavender (#a082e6) in the mist over Saltsjön; warm amber window slit; Djurgården silhouette in near-black (#34303d); the lake mirrors all colors one shade darker. Slow dolly back; the sauna shrinks; Djurgården and the harbor entrance reveal themselves; the dawn sky brightens; the bird crosses; mist wisps drift off Saltsjön; the fire glow flickers its last.</t>
   </si>
   <si>
@@ -1528,81 +1532,109 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="15" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="18"/>
       <color rgb="FF2E008B"/>
-      <sz val="18"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="12"/>
       <color rgb="FF9B0AA5"/>
-      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="14"/>
       <color rgb="FF2E008B"/>
-      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF34303D"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FF9B0AA5"/>
-      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF34303D"/>
-      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FF2E008B"/>
-      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FF34303D"/>
-      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="16"/>
       <color rgb="FF2E008B"/>
-      <sz val="16"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
+      <sz val="9"/>
       <color rgb="FF9B0AA5"/>
-      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="16"/>
       <color rgb="FF9B0AA5"/>
-      <sz val="16"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="16"/>
       <color rgb="FF3750DC"/>
-      <sz val="16"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FF3750DC"/>
-      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -2132,19 +2164,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FF2E008B"/>
   </sheetPr>
   <dimension ref="A1:C33"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2152,7 +2184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2160,7 +2192,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -2168,7 +2200,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -2179,7 +2211,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -2190,7 +2222,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -2201,7 +2233,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -2212,7 +2244,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -2223,7 +2255,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -2231,7 +2263,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="60" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -2242,7 +2274,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -2250,7 +2282,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -2261,7 +2293,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -2272,7 +2304,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -2283,7 +2315,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -2294,7 +2326,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -2305,7 +2337,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -2316,7 +2348,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>0</v>
       </c>
@@ -2327,7 +2359,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -2338,7 +2370,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -2349,7 +2381,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>0</v>
       </c>
@@ -2360,7 +2392,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>0</v>
       </c>
@@ -2373,17 +2405,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FFA082E6"/>
   </sheetPr>
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -2395,17 +2427,17 @@
     <col min="8" max="8" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
         <v>42</v>
       </c>
@@ -2431,7 +2463,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A5" s="14">
         <v>1</v>
       </c>
@@ -2457,7 +2489,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="255" x14ac:dyDescent="0.2">
       <c r="A6" s="17">
         <v>2</v>
       </c>
@@ -2483,7 +2515,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="210" x14ac:dyDescent="0.2">
       <c r="A7" s="14">
         <v>3</v>
       </c>
@@ -2509,7 +2541,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A8" s="17">
         <v>4</v>
       </c>
@@ -2535,7 +2567,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="210" x14ac:dyDescent="0.2">
       <c r="A9" s="14">
         <v>5</v>
       </c>
@@ -2561,7 +2593,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="255" x14ac:dyDescent="0.2">
       <c r="A10" s="17">
         <v>6</v>
       </c>
@@ -2587,7 +2619,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="210" x14ac:dyDescent="0.2">
       <c r="A11" s="14">
         <v>7</v>
       </c>
@@ -2613,7 +2645,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A12" s="17">
         <v>8</v>
       </c>
@@ -2639,7 +2671,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="210" x14ac:dyDescent="0.2">
       <c r="A13" s="14">
         <v>9</v>
       </c>
@@ -2665,7 +2697,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A14" s="17">
         <v>10</v>
       </c>
@@ -2691,7 +2723,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="210" x14ac:dyDescent="0.2">
       <c r="A15" s="14">
         <v>11</v>
       </c>
@@ -2717,7 +2749,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A16" s="17">
         <v>12</v>
       </c>
@@ -2743,7 +2775,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="210" x14ac:dyDescent="0.2">
       <c r="A17" s="14">
         <v>13</v>
       </c>
@@ -2769,7 +2801,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="210" x14ac:dyDescent="0.2">
       <c r="A18" s="17">
         <v>14</v>
       </c>
@@ -2795,7 +2827,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A19" s="14">
         <v>15</v>
       </c>
@@ -2821,7 +2853,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A20" s="17">
         <v>16</v>
       </c>
@@ -2847,7 +2879,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="210" x14ac:dyDescent="0.2">
       <c r="A21" s="14">
         <v>17</v>
       </c>
@@ -2873,7 +2905,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A22" s="17">
         <v>18</v>
       </c>
@@ -2899,7 +2931,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A23" s="14">
         <v>19</v>
       </c>
@@ -2925,7 +2957,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A24" s="17">
         <v>20</v>
       </c>
@@ -2951,7 +2983,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A25" s="14">
         <v>21</v>
       </c>
@@ -2977,7 +3009,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A26" s="17">
         <v>22</v>
       </c>
@@ -3003,7 +3035,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A27" s="14">
         <v>23</v>
       </c>
@@ -3029,7 +3061,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A28" s="17">
         <v>24</v>
       </c>
@@ -3055,7 +3087,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="285" x14ac:dyDescent="0.2">
       <c r="A29" s="14">
         <v>25</v>
       </c>
@@ -3082,19 +3114,19 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H4"/>
+  <autoFilter ref="A4:H4" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FFEB5ADC"/>
   </sheetPr>
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -3106,17 +3138,17 @@
     <col min="8" max="8" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="21" t="s">
         <v>42</v>
       </c>
@@ -3142,7 +3174,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="210" x14ac:dyDescent="0.2">
       <c r="A5" s="22">
         <v>1</v>
       </c>
@@ -3168,7 +3200,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A6" s="24">
         <v>2</v>
       </c>
@@ -3194,7 +3226,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A7" s="22">
         <v>3</v>
       </c>
@@ -3220,7 +3252,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A8" s="24">
         <v>4</v>
       </c>
@@ -3246,7 +3278,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A9" s="22">
         <v>5</v>
       </c>
@@ -3272,7 +3304,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A10" s="24">
         <v>6</v>
       </c>
@@ -3298,7 +3330,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A11" s="22">
         <v>7</v>
       </c>
@@ -3324,7 +3356,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A12" s="24">
         <v>8</v>
       </c>
@@ -3350,7 +3382,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="210" x14ac:dyDescent="0.2">
       <c r="A13" s="22">
         <v>9</v>
       </c>
@@ -3376,7 +3408,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A14" s="24">
         <v>10</v>
       </c>
@@ -3402,7 +3434,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A15" s="22">
         <v>11</v>
       </c>
@@ -3428,7 +3460,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A16" s="24">
         <v>12</v>
       </c>
@@ -3454,7 +3486,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A17" s="22">
         <v>13</v>
       </c>
@@ -3480,7 +3512,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A18" s="24">
         <v>14</v>
       </c>
@@ -3506,7 +3538,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A19" s="22">
         <v>15</v>
       </c>
@@ -3532,7 +3564,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A20" s="24">
         <v>16</v>
       </c>
@@ -3558,7 +3590,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A21" s="22">
         <v>17</v>
       </c>
@@ -3584,7 +3616,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A22" s="24">
         <v>18</v>
       </c>
@@ -3610,7 +3642,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A23" s="22">
         <v>19</v>
       </c>
@@ -3636,7 +3668,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A24" s="24">
         <v>20</v>
       </c>
@@ -3662,7 +3694,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A25" s="22">
         <v>21</v>
       </c>
@@ -3688,7 +3720,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A26" s="24">
         <v>22</v>
       </c>
@@ -3714,7 +3746,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A27" s="22">
         <v>23</v>
       </c>
@@ -3740,7 +3772,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A28" s="24">
         <v>24</v>
       </c>
@@ -3766,7 +3798,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A29" s="22">
         <v>25</v>
       </c>
@@ -3793,19 +3825,19 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H4"/>
+  <autoFilter ref="A4:H4" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor rgb="FF7DA0EB"/>
   </sheetPr>
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -3817,17 +3849,17 @@
     <col min="8" max="8" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="27" t="s">
         <v>42</v>
       </c>
@@ -3853,7 +3885,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A5" s="28">
         <v>1</v>
       </c>
@@ -3879,7 +3911,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A6" s="30">
         <v>2</v>
       </c>
@@ -3905,7 +3937,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A7" s="28">
         <v>3</v>
       </c>
@@ -3931,7 +3963,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A8" s="30">
         <v>4</v>
       </c>
@@ -3957,7 +3989,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A9" s="28">
         <v>5</v>
       </c>
@@ -3983,7 +4015,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A10" s="30">
         <v>6</v>
       </c>
@@ -4009,7 +4041,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A11" s="28">
         <v>7</v>
       </c>
@@ -4035,7 +4067,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A12" s="30">
         <v>8</v>
       </c>
@@ -4061,7 +4093,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="255" x14ac:dyDescent="0.2">
       <c r="A13" s="28">
         <v>9</v>
       </c>
@@ -4087,7 +4119,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="285" x14ac:dyDescent="0.2">
       <c r="A14" s="30">
         <v>10</v>
       </c>
@@ -4113,7 +4145,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A15" s="28">
         <v>11</v>
       </c>
@@ -4139,7 +4171,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A16" s="30">
         <v>12</v>
       </c>
@@ -4165,7 +4197,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A17" s="28">
         <v>13</v>
       </c>
@@ -4191,7 +4223,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="225" x14ac:dyDescent="0.2">
       <c r="A18" s="30">
         <v>14</v>
       </c>
@@ -4217,7 +4249,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="285" x14ac:dyDescent="0.2">
       <c r="A19" s="28">
         <v>15</v>
       </c>
@@ -4243,7 +4275,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A20" s="30">
         <v>16</v>
       </c>
@@ -4269,7 +4301,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A21" s="28">
         <v>17</v>
       </c>
@@ -4295,7 +4327,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A22" s="30">
         <v>18</v>
       </c>
@@ -4321,7 +4353,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="240" x14ac:dyDescent="0.2">
       <c r="A23" s="28">
         <v>19</v>
       </c>
@@ -4347,7 +4379,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="255" x14ac:dyDescent="0.2">
       <c r="A24" s="30">
         <v>20</v>
       </c>
@@ -4373,7 +4405,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="285" x14ac:dyDescent="0.2">
       <c r="A25" s="28">
         <v>21</v>
       </c>
@@ -4399,7 +4431,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="255" x14ac:dyDescent="0.2">
       <c r="A26" s="30">
         <v>22</v>
       </c>
@@ -4425,7 +4457,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="270" x14ac:dyDescent="0.2">
       <c r="A27" s="28">
         <v>23</v>
       </c>
@@ -4451,7 +4483,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="255" x14ac:dyDescent="0.2">
       <c r="A28" s="30">
         <v>24</v>
       </c>
@@ -4477,7 +4509,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="300" x14ac:dyDescent="0.2">
       <c r="A29" s="28">
         <v>25</v>
       </c>
@@ -4504,8 +4536,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H4"/>
+  <autoFilter ref="A4:H4" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>